<commit_message>
Add Telegram-verified quiz answers
</commit_message>
<xml_diff>
--- a/Simple_Quiz_Intelligence_v1_rebuilt.xlsx
+++ b/Simple_Quiz_Intelligence_v1_rebuilt.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Каталог" sheetId="1" r:id="R0fe8e1ef71fa4e17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Механики" sheetId="2" r:id="R2f9893658a9a46be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Раунды" sheetId="3" r:id="R8df6ad2b5b3147c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дашборд" sheetId="4" r:id="R069312a83ec84449"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Новые пакеты" sheetId="5" r:id="R24597f7720f04c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram-архив" sheetId="6" r:id="R94212dc32542464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Каталог" sheetId="1" r:id="R2fc779dd31c543cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Механики" sheetId="2" r:id="Re8647745720143a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Раунды" sheetId="3" r:id="R195218a2d7fe47bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дашборд" sheetId="4" r:id="Rc8b75b4f86b44b76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Новые пакеты" sheetId="5" r:id="R8e8e1aedc90242b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram-архив" sheetId="6" r:id="Rca472f345e024a4c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -426,7 +426,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1af9194eaac94625"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdfbec3e15ba947cf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2908,7 +2908,7 @@
         <x:v>Этот сезон НХЛ - уникальный: домашний матч «Каролины» против «Тампа-Бэй» перенесли из-за НЕГО, а матч «Лос-Анджелеса» против «Калгари» перенесли из-за НИХ. Как иронично. Назовите ЕГО и ИХ.</x:v>
       </x:c>
       <x:c r="F50" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Ураган и пожары</x:v>
       </x:c>
       <x:c r="G50" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -2917,7 +2917,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I50" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/6?comment=6</x:v>
       </x:c>
       <x:c r="J50" s="6"/>
       <x:c r="K50" s="6" t="str">
@@ -2948,7 +2948,7 @@
         <x:v>Если ты любитель спорта, то в Америке тебе не удастся сходить на рэп, поп или фолк, зато можно сходить на рок, на ИКС и на ИГРЕК. Назовите ИКС и ИГРЕК. о</x:v>
       </x:c>
       <x:c r="F51" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>«Юта Джаз» и «Сент-Луис Блюз»</x:v>
       </x:c>
       <x:c r="G51" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -2957,7 +2957,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I51" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/7?comment=10</x:v>
       </x:c>
       <x:c r="J51" s="6"/>
       <x:c r="K51" s="6" t="str">
@@ -2988,7 +2988,7 @@
         <x:v>Рядом с ЭТИМ на футбольных матчах с 2020 года красуется цифра 5, с 2013 года - 4, с 2006 года - 3, с 2000 года - 2. А вообще ЭТО фигурирует в трансляциях некоторых футбольных матчей с 1995 года. О чем речь?</x:v>
       </x:c>
       <x:c r="F52" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>PS (PlayStation)</x:v>
       </x:c>
       <x:c r="G52" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -2997,7 +2997,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I52" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/17?comment=27</x:v>
       </x:c>
       <x:c r="J52" s="6"/>
       <x:c r="K52" s="6" t="str">
@@ -3028,7 +3028,7 @@
         <x:v>Первая ОНА появились в России в 2001 году. Сейчас ИХ более 40 в Москве и Московской области. Ав 2018 году благодаря паре русских футболистов одна из НИХ на протяжении нескольких месяцев регулярно появлялась в новостных каналах и пабликах. Назовите EE.</x:v>
       </x:c>
       <x:c r="F53" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кофемания</x:v>
       </x:c>
       <x:c r="G53" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3037,7 +3037,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I53" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/19?comment=30</x:v>
       </x:c>
       <x:c r="J53" s="6"/>
       <x:c r="K53" s="6" t="str">
@@ -3148,7 +3148,7 @@
         <x:v>В 2014 году 21-летняя испанка Гарбинье Мугуруса сенсационно выбила из сетки «Ролан Гаррос» Серену Уильямс и добралась до до четвертьфинала турнира «Большого шлема». На сайте Eurosport.ru вышел пост с фактами про Гарбинье. Назывался он так: «Мугуруса, ПРОПУСК». Заголовок - аллюзия на популярную в середине 20 века фразу: она не раз звучала в самом известном фильме про пионеров. Какие два слова мы пропустили в заголовке текста на Eurosport.ru?</x:v>
       </x:c>
       <x:c r="F56" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>А что вы тут делаете, а?</x:v>
       </x:c>
       <x:c r="G56" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3157,7 +3157,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I56" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/127?comment=223</x:v>
       </x:c>
       <x:c r="J56" s="6"/>
       <x:c r="K56" s="6" t="str">
@@ -3188,7 +3188,7 @@
         <x:v>Было бы символично, если бы ИКС ИГРЕК играл за ЗЕТ ИКС, но нет: в США он выступал лишь за одну команду. Назовите ИКС. Если вы знаете, что за песня Queen играла в рекламе Coca-Cola, вам, скорее всего, будет проще справиться с этим вопросом.</x:v>
       </x:c>
       <x:c r="F57" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мэджик</x:v>
       </x:c>
       <x:c r="G57" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3197,7 +3197,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I57" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/130?comment=239</x:v>
       </x:c>
       <x:c r="J57" s="6"/>
       <x:c r="K57" s="6" t="str">
@@ -3228,7 +3228,7 @@
         <x:v>ЭТО есть как минимум в двух экземплярах у каждого профессионального клуба. ЭТО было и в названии одного из клубов НБА, нос 2012 года не фигурирует в нем. О чем речь?</x:v>
       </x:c>
       <x:c r="F58" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Джерси</x:v>
       </x:c>
       <x:c r="G58" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3237,7 +3237,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I58" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/141?comment=252</x:v>
       </x:c>
       <x:c r="J58" s="6"/>
       <x:c r="K58" s="6" t="str">
@@ -3268,7 +3268,7 @@
         <x:v>Назовите команду МФЛ, которая всегда располагается в таблице на 22-м месте.</x:v>
       </x:c>
       <x:c r="F59" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Титан</x:v>
       </x:c>
       <x:c r="G59" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3277,7 +3277,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I59" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/142?comment=255</x:v>
       </x:c>
       <x:c r="J59" s="6"/>
       <x:c r="K59" s="6" t="str">
@@ -3348,7 +3348,7 @@
         <x:v>Этот оскорбительный термин применительно к девушкам регулярно вспоминают в русскоязычном твиттере. В одном из олимпийских видов спорта так можно безоценочно назвать его представительниц. Среди олимпийских чемпионок в этом виде спорта в 21 веке - чилийка Франсиска Кроветто, американки Эмбер Инглиш и Ким Роуд, итальянки Диана Бакози и Кьяра Кайнеро, венгерка Диана Игали. Наверное, несправедливо, что некоторым из вас официанты принесли подсказку. Назовите этот термин.</x:v>
       </x:c>
       <x:c r="F61" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тарелочница</x:v>
       </x:c>
       <x:c r="G61" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3357,7 +3357,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I61" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/157?comment=364</x:v>
       </x:c>
       <x:c r="J61" s="6"/>
       <x:c r="K61" s="6" t="str">
@@ -3388,7 +3388,7 @@
         <x:v>Валентин Серов посвятил краже ИКС не одно полотно: говорят, он написал шесть вариантов картины. Карло Анчелотти вызвал 25 футболистов на первые для него у руля матчи сборной Бразилии. Четыре из них никогда не играли в ИКС. Несмотря на то, что технически вы в ИКС прямо сейчас, некоторые из вас могут похвастаться, что были в ИКС. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F62" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Европа</x:v>
       </x:c>
       <x:c r="G62" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3397,7 +3397,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I62" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/178?comment=423</x:v>
       </x:c>
       <x:c r="J62" s="6"/>
       <x:c r="K62" s="6" t="str">
@@ -3428,7 +3428,7 @@
         <x:v>В конце 15 века итальянский художник написал картину, на которой было изображено первое событие в жизни АЛЬФЫ. Картина была написана по заказу представителя семьи Медичи. Полотно до сих пор хранится в галерее Уффици. 17 июня 1980 года произошло первое событие в жизни другой АЛЬФЫ. Напишите в ответе название картины.</x:v>
       </x:c>
       <x:c r="F63" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>«Рождение Венеры»</x:v>
       </x:c>
       <x:c r="G63" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3437,7 +3437,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I63" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/180?comment=451</x:v>
       </x:c>
       <x:c r="J63" s="6"/>
       <x:c r="K63" s="6" t="str">
@@ -3468,7 +3468,7 @@
         <x:v>В английском языке это слово означает близкого друга, братишку. Если это же слово написать кириллицей, получится некое действие во множественном числе, свидетелем которого можно стать, например, в петанке, дартсе и водном поло. Напишите это слово кириллицей.</x:v>
       </x:c>
       <x:c r="F64" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Броски</x:v>
       </x:c>
       <x:c r="G64" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3477,7 +3477,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I64" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/181?comment=459</x:v>
       </x:c>
       <x:c r="J64" s="6"/>
       <x:c r="K64" s="6" t="str">
@@ -3508,7 +3508,7 @@
         <x:v>У группы Oasis и рэпера Big Baby Tape есть треки с одинаковым названием. Увидев название этих треков, в голову сразу приходит важный для истории НБА город. О каком городе речь?</x:v>
       </x:c>
       <x:c r="F65" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сиэтл</x:v>
       </x:c>
       <x:c r="G65" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3517,7 +3517,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I65" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/187?comment=485</x:v>
       </x:c>
       <x:c r="J65" s="6"/>
       <x:c r="K65" s="6" t="str">
@@ -3548,7 +3548,7 @@
         <x:v>Российского предпринимателя из Троицка, который открыл бизнес в Сыктывкаре, и линию обороны футбольного клуба «Рома» с 2012 по 2014. год, объединяют два повторяющихся слога. Напишите эти два одинаковых слога.</x:v>
       </x:c>
       <x:c r="F66" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Додо</x:v>
       </x:c>
       <x:c r="G66" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3557,7 +3557,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I66" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/206?comment=535</x:v>
       </x:c>
       <x:c r="J66" s="6"/>
       <x:c r="K66" s="6" t="str">
@@ -3628,7 +3628,7 @@
         <x:v>В 2019 году в сторисах Sports.ru провели небольшой квиз из трех картинок. На первой была показана картина «Впечатление». Вопрос на картинке был следующим: «Это шедевр ИКСА?» Правильный ответ, конечно, — «Нет». На второй тот же вопрос с тем же ответом дали рядом с картиной «Олимпия». На третьей была фотография из матча «Ливерпуль» - «Бавария». Вопрос на картинке совпадал: «Это шедевр ИКСА?» Правильный ответ - «Да!» В ЛЧ-2018/19 ИКС забил 4 гола. Назовите ИКС двумя словами.</x:v>
       </x:c>
       <x:c r="F68" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Садио Мане</x:v>
       </x:c>
       <x:c r="G68" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3637,7 +3637,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I68" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/213?comment=553</x:v>
       </x:c>
       <x:c r="J68" s="6"/>
       <x:c r="K68" s="6" t="str">
@@ -3708,7 +3708,7 @@
         <x:v>В треке Carefree, вышедшем в 2021 году, рэпер Songer занеймдроппил очень много футболистов. В одной из строчек он говорит, что у «Манчестер Сити» есть Рахим Стерлинг, но нет страйкера, поэтому клуб из Манчестера хочет ЕГО. За кем, по мнению Songer, охотился «Сити»?</x:v>
       </x:c>
       <x:c r="F70" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Эрлинг Холанд</x:v>
       </x:c>
       <x:c r="G70" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3717,7 +3717,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I70" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/251?comment=645</x:v>
       </x:c>
       <x:c r="J70" s="6"/>
       <x:c r="K70" s="6" t="str">
@@ -3748,7 +3748,7 @@
         <x:v>По состоянию на 2025 год Израиль, Кипр и Армения - единственные члены УЕФА, у которых нет ЭТОГО. О чем речь?</x:v>
       </x:c>
       <x:c r="F71" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Нахождение на территории Европы</x:v>
       </x:c>
       <x:c r="G71" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3757,7 +3757,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I71" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/261?comment=669</x:v>
       </x:c>
       <x:c r="J71" s="6"/>
       <x:c r="K71" s="6" t="str">
@@ -3788,7 +3788,7 @@
         <x:v>В сезоне-2025/26 в АПЛ их 7, в Чемпионшипе — 3, в английской Лиге 1 - 2, ав Лиге 2-1. О чем речь?</x:v>
       </x:c>
       <x:c r="F72" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Клубы из Лондона</x:v>
       </x:c>
       <x:c r="G72" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3797,7 +3797,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I72" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/262?comment=667</x:v>
       </x:c>
       <x:c r="J72" s="6"/>
       <x:c r="K72" s="6" t="str">
@@ -3828,7 +3828,7 @@
         <x:v>829 7” Sf о® Этот футболист провел всего год в «Дженоз», а потом укатил в Англию и следующие 8 лет играл исключительно в английских клубах. По окончании карьеры он тренировал клубы из восьми разных стран (и, в частности, работал в двух командах РПЛ). Аниме, в названии которого аж дважды содержится имя этого футболиста, прямо сейчас можно посмотреть в «Амедиатеке», а первые серии второго сезона летом показывали в московских кинотеатрах. Назовите этого футболиста. т WIN BOX od</x:v>
       </x:c>
       <x:c r="F73" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Дан Петреску</x:v>
       </x:c>
       <x:c r="G73" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3837,7 +3837,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I73" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/263?comment=673</x:v>
       </x:c>
       <x:c r="J73" s="6"/>
       <x:c r="K73" s="6" t="str">
@@ -3868,7 +3868,7 @@
         <x:v>9 2? Sf o° P Если записать названия клубов Ла Лиги с помощью элементов периодической таблицы, это получится с «Осасуной» (Os, As, Ц, Ма), «Бетисом» (Re, Al, Be, Ti, $) иеще одним клубом. В 2020 году этот клуб на один матч убрал из своего названия 4 буквы, оставив лишь Te, что с испанского переводятся как «вера», а в периодической таблице находятся на 26-м месте. Назовите этот клуб. — WIN вох ool</x:v>
       </x:c>
       <x:c r="F74" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Хетафе</x:v>
       </x:c>
       <x:c r="G74" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3877,7 +3877,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I74" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/264?comment=681</x:v>
       </x:c>
       <x:c r="J74" s="6"/>
       <x:c r="K74" s="6" t="str">
@@ -3908,7 +3908,7 @@
         <x:v>9 2? ve Va A о® АЛЬФА - вещь, которую видел или даже держал в руках каждый из вас. Один килограмм вяленых АЛЬФ можно найти на маркетплейсах за 3500 рублей, в то же время мешок АЛЬФ оценивают всего в 500 рублей. АЛЬФУ можно найти и на эмблеме одного из клубов Бундеслиги. Понять, какая именно АЛЬФА на эмблеме, просто: небольшой размер, округлая форма и направление вверх. Назовите АЛЬФУ. ее cnunmnn WIN BOX ool</x:v>
       </x:c>
       <x:c r="F75" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кедровая шишка</x:v>
       </x:c>
       <x:c r="G75" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3917,7 +3917,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I75" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/265?comment=688</x:v>
       </x:c>
       <x:c r="J75" s="6"/>
       <x:c r="K75" s="6" t="str">
@@ -3948,7 +3948,7 @@
         <x:v>Надпись на футболке этого футболиста в зависимости от эпохи и культурного контекста может означать как устройство для воспроизведения видео, так и последовательность чисел 5, 1, 500, 1, 100. Назовите этого футболиста.</x:v>
       </x:c>
       <x:c r="F76" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Неманья Видич</x:v>
       </x:c>
       <x:c r="G76" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3957,7 +3957,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I76" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/285?comment=737</x:v>
       </x:c>
       <x:c r="J76" s="6"/>
       <x:c r="K76" s="6" t="str">
@@ -4028,7 +4028,7 @@
         <x:v>ОМЕГА - локально культовый российский спортсмен не только благодаря результатам, но и благодаря ассоциации с трехзначным четным числом. Как только ты захотел спеть или сыграть музыкальное произведение с кем-то, ОМЕГА перестает быть ОМЕГОИ. Назовите ОМЕГУ.</x:v>
       </x:c>
       <x:c r="F78" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Соло 322</x:v>
       </x:c>
       <x:c r="G78" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4037,7 +4037,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I78" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/291?comment=760</x:v>
       </x:c>
       <x:c r="J78" s="6"/>
       <x:c r="K78" s="6" t="str">
@@ -4068,7 +4068,7 @@
         <x:v>Песня с названием «ИКС» вышла на альбоме 1999 года. 19 лет спустя та же группа выпустила песню «В ИКСЕ». Поклонники ИКСА поют ее на трибунах намного чаще. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F79" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Зенит</x:v>
       </x:c>
       <x:c r="G79" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4077,7 +4077,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I79" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/294?comment=772</x:v>
       </x:c>
       <x:c r="J79" s="6"/>
       <x:c r="K79" s="6" t="str">
@@ -4108,7 +4108,7 @@
         <x:v>Из некоторых сокращений команд НХЛ получается слово на английском. Так, сокращение «Питтсбурга» — PIT — переводится как «яма», а сокращение «Сиэтла» - SEA - переводится как «море». Сокращения сразу двух клубов НХЛ в переводе означают транспортные средства. Назовите эти транспортные средства.</x:v>
       </x:c>
       <x:c r="F80" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Car и van</x:v>
       </x:c>
       <x:c r="G80" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4117,7 +4117,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I80" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/301?comment=788</x:v>
       </x:c>
       <x:c r="J80" s="6"/>
       <x:c r="K80" s="6" t="str">
@@ -4148,7 +4148,7 @@
         <x:v>В стандартной клавиатуре Windows 104 клавиши. Одна из них практически не используется в играх — в том числе и в той серии, название которой иллюстрирует. Например, в версии видеоигры 2021 года этой клавиши не было, а в версии 2025 года она по умолчанию обозначала «Extra Action 1». О какой клавише речь?</x:v>
       </x:c>
       <x:c r="F81" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="G81" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4157,7 +4157,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I81" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/302?comment=791</x:v>
       </x:c>
       <x:c r="J81" s="6"/>
       <x:c r="K81" s="6" t="str">
@@ -4188,7 +4188,7 @@
         <x:v>Псевдоним этого инди-исполнителя состоит из трех слов. Последние два описывают процесс, первое — ИКС: мужское имя в уменьшительной форме. Один из его самых популярных треков - «Волна». Также ИКС - разговорный синоним слова «команда». Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F82" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тима</x:v>
       </x:c>
       <x:c r="G82" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4197,7 +4197,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I82" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/320?comment=821</x:v>
       </x:c>
       <x:c r="J82" s="6"/>
       <x:c r="K82" s="6" t="str">
@@ -4228,7 +4228,7 @@
         <x:v>В 2022 году Василий Уткин говорил, что по утрам он обычно писал тексты, смотрел кино и даже делал зарядку. «Вы, наверное, удивитесь, но у меня дома есть ОНИ. И я ими пользуюсь по назначению», — рассказывал Василий. В отличие отлирического героя группы «Кровосток»: он пользовался ЕЙ не по назначению.</x:v>
       </x:c>
       <x:c r="F83" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Гантели</x:v>
       </x:c>
       <x:c r="G83" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4237,7 +4237,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I83" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/321?comment=825</x:v>
       </x:c>
       <x:c r="J83" s="6"/>
       <x:c r="K83" s="6" t="str">
@@ -4308,7 +4308,7 @@
         <x:v>В матчах ЦСКА можно стать свидетелем математического оксюморона. Его можно описать словосочетанием «ИКС ИГРЕКА». ИКС - часть фанатского сленга, а ИГРЕК - прозвище одного из футболистов ЦСКА. Назовите словосочетание, которое мы загадали.</x:v>
       </x:c>
       <x:c r="F85" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Угол круга</x:v>
       </x:c>
       <x:c r="G85" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4317,7 +4317,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I85" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/326?comment=843</x:v>
       </x:c>
       <x:c r="J85" s="6"/>
       <x:c r="K85" s="6" t="str">
@@ -4348,7 +4348,7 @@
         <x:v>Все мы подписываемся на блогеров или медиа в надежде получить кое-что качественное. ЭТОТ ИГРОК отличается от кое-чего наличием одной гласной буквы. Был ли ОН качественным - = вопрос дискуссионный, но 69 матчей за © 7 «Баварию» и 94 - за «Бордо» он провел О каком игроке идет речь? = i</x:v>
       </x:c>
       <x:c r="F86" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Контенто</x:v>
       </x:c>
       <x:c r="G86" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4357,7 +4357,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I86" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/327?comment=847</x:v>
       </x:c>
       <x:c r="J86" s="6"/>
       <x:c r="K86" s="6" t="str">
@@ -4388,7 +4388,7 @@
         <x:v>ИКС - российский бренд, который существует с 1995 года. Он специализируется на кетчупах, томатных пастах и уксусах. Сходить на ИКС у вас получится в НФЛ и MLB и не получится - в НХЛ, НБА и MLS. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F87" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Балтимор</x:v>
       </x:c>
       <x:c r="G87" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4397,7 +4397,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I87" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/330?comment=851</x:v>
       </x:c>
       <x:c r="J87" s="6"/>
       <x:c r="K87" s="6" t="str">
@@ -4508,7 +4508,7 @@
         <x:v>Когда хоккеиста Максима Афиногенова спросили про АЛЬФЫ, которые летят на лед во время матчей его команды, он ответил, что подобное встречается и в НХЛ, и привел пример с традицией в «Детройте» кидать на лед осьминога. Правда, если осьминог для «Ред Уингс» — победный символ, то АЛЬФА - оскорбление конкретной команды. Про что спросили после матча Макса Афиногенова?</x:v>
       </x:c>
       <x:c r="F90" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сосиски</x:v>
       </x:c>
       <x:c r="G90" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4517,7 +4517,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I90" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/355?comment=906</x:v>
       </x:c>
       <x:c r="J90" s="6"/>
       <x:c r="K90" s="6" t="str">
@@ -4548,7 +4548,7 @@
         <x:v>Несколько лет назад в интернете стало вирусным изображение одного ИКСа и Криштиану Роналду. Глядя на него, трудно поверить, что «ОМЕГА» ИКСА случилось позже - примерно через 308 дней после Роналду и через 474. года после «ОМЕГИ ИКСА» Микеланджело. Назовите, что такое ОМЕГА ИКСА.</x:v>
       </x:c>
       <x:c r="F91" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>«Сотворение Адама»</x:v>
       </x:c>
       <x:c r="G91" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4557,7 +4557,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I91" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/356?comment=913</x:v>
       </x:c>
       <x:c r="J91" s="6"/>
       <x:c r="K91" s="6" t="str">
@@ -4588,7 +4588,7 @@
         <x:v>Основное время семи матчей ЧМ-2018 закончилось со счетом, который можно записать, используя лишь имя одного из древних богов. Один из этих семи матчей, уверен, смотрел практически каждый из вас. Напишите счет этих матчей, используя лишь имя бога, но столько раз, сколько посчитаете нужным.</x:v>
       </x:c>
       <x:c r="F92" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>1:1</x:v>
       </x:c>
       <x:c r="G92" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4597,7 +4597,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I92" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/367?comment=931</x:v>
       </x:c>
       <x:c r="J92" s="6"/>
       <x:c r="K92" s="6" t="str">
@@ -4628,7 +4628,7 @@
         <x:v>С середины 2010-х несложно получить ретвит от одного из комментаторов Eurosport: достаточно сфотографировать автомобиль с этим трехзначным номером и отметить одного из комментаторов. Он почти всегда ретвитит фото с подобными номерами. Назовите трехзначное число, о котором мы рассказали в предыдущем абзаце.</x:v>
       </x:c>
       <x:c r="F93" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="G93" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4637,7 +4637,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I93" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/371?comment=966</x:v>
       </x:c>
       <x:c r="J93" s="6"/>
       <x:c r="K93" s="6" t="str">
@@ -4668,7 +4668,7 @@
         <x:v>На «Википедии» можно найти свыше 30 различных ИКСОВ: это, например, и город в Калифорнии, и столица острова Тенерифе, и крупнейший город Боливии. Но мы помним другого ИКСА: того, что играл за «Баварию», «Манчестер Сити», «Блэкберн», «Малагу» и «Бетис». А еще - за мексиканский клуб, название которого ну очень ему подходит. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F94" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Санта-Крус</x:v>
       </x:c>
       <x:c r="G94" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4677,7 +4677,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I94" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/374?comment=976</x:v>
       </x:c>
       <x:c r="J94" s="6"/>
       <x:c r="K94" s="6" t="str">
@@ -4748,7 +4748,7 @@
         <x:v>ИКС - экс-футболист «Зенита», который, помимо России, поиграл в Германии, Греции, Турции, Венгрии и даже Австралии. ИКСЫ - картина Винсента ван Гога 1887 года. Кстати, в период карьеры в «Зените» у ИКСА не было на спине ни единицы, ни восьмерки, ни семерки. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F96" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мак</x:v>
       </x:c>
       <x:c r="G96" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4757,7 +4757,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I96" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/388?comment=1007</x:v>
       </x:c>
       <x:c r="J96" s="6"/>
       <x:c r="K96" s="6" t="str">
@@ -4788,7 +4788,7 @@
         <x:v>Один ИКС изначально был не ИКСОМ, а Чейни. Другой ИКС раньше был не ИКСОМ, а Августой. Один ИКС периодически зарабатывал деньги боксом. Другой ИКС не раз принимал крупные боксерские поединки. Там дрались и Поветкин, и Кличко. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F97" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лондон</x:v>
       </x:c>
       <x:c r="G97" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4797,7 +4797,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I97" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/392?comment=1025</x:v>
       </x:c>
       <x:c r="J97" s="6"/>
       <x:c r="K97" s="6" t="str">
@@ -4828,7 +4828,7 @@
         <x:v>Всю карьеру ОН выступал на резине бренда Light Year. В числе его спонсоров - Vitoline, Clutch+Aid, Mood Springs, Octane Gain, NitroAde, Easy Idle. Логотипы этих брендов можно увидеть Ha HEM. Назовите ЕГО двумя словами.</x:v>
       </x:c>
       <x:c r="F98" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Молния Маккуин</x:v>
       </x:c>
       <x:c r="G98" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4837,7 +4837,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I98" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/399?comment=1043</x:v>
       </x:c>
       <x:c r="J98" s="6"/>
       <x:c r="K98" s="6" t="str">
@@ -4868,7 +4868,7 @@
         <x:v>Аккаунт nbaresdev выяснил, что игроки НБА начинают играть хуже после того, как обзаводятся ИМИ. В качестве доказательства они привели статистику Леброна Джеймса, Кевина Дюранта, Дреймонда Грина, Пола Джорджаи Джей Джея Редика. У всех них упали цифры по сезону после появления ИХ в их жизни. По одной из версий, первый ОН появился в 2004 году. В том же году это слово впервые использовал журналист Бен Хаммерсли. Кого мы зашифровали под НИМ?</x:v>
       </x:c>
       <x:c r="F99" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Подкаст</x:v>
       </x:c>
       <x:c r="G99" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4877,7 +4877,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I99" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/415?comment=1083</x:v>
       </x:c>
       <x:c r="J99" s="6"/>
       <x:c r="K99" s="6" t="str">
@@ -4908,7 +4908,7 @@
         <x:v>Американская актриса Оливия Коберн известна многим из вас под другой фамилией. Одна из самых популярных сериальных ролей Оливии - ИКС. Догадаться, что мы спрятали под ИКСОМ, вам помогут Микаэль Баллак, Алессандро Неста и Майкон. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F100" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тринадцатая</x:v>
       </x:c>
       <x:c r="G100" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4917,7 +4917,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I100" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/417?comment=1098</x:v>
       </x:c>
       <x:c r="J100" s="6"/>
       <x:c r="K100" s="6" t="str">
@@ -4948,7 +4948,7 @@
         <x:v>Бенджамин Франклин говорил, что не наблюдать за ИКСАМИ - значит, оставлять им открытым свой кошелек. Если к ИКСАМ добавить согласную букву, получится название футбольного клуба, который в августе 2005 года приезжал в Москву на матч с «Локомотивом». Назовите этот клуб.</x:v>
       </x:c>
       <x:c r="F101" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Работнички</x:v>
       </x:c>
       <x:c r="G101" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4957,7 +4957,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I101" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/418?comment=1103</x:v>
       </x:c>
       <x:c r="J101" s="6"/>
       <x:c r="K101" s="6" t="str">
@@ -4988,7 +4988,7 @@
         <x:v>В 1978-1979 годах логотип «Нью-Йорк Никс» был в форме НЕГО. Вот некоторые ИХ представители: Fuji, Empire, Jonathan, Arkansas Black, Discovery. О чем речь?</x:v>
       </x:c>
       <x:c r="F102" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Яблоко</x:v>
       </x:c>
       <x:c r="G102" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -4997,7 +4997,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I102" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/421?comment=1112</x:v>
       </x:c>
       <x:c r="J102" s="6"/>
       <x:c r="K102" s="6" t="str">
@@ -5028,7 +5028,7 @@
         <x:v>В ноябре 2022 года в соревновательный Counter-Strike добавили ИКС. Правда, уже через пару лет его убрали из про-сцены. Вы могли слышать про ИКСА на уроках истории. Если бы вы назвали ИКСА шакалом, это в какой-то степени было правдивым утверждением. В одной из древних культур он считался изобретателем бальзамирования. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F103" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Анубис</x:v>
       </x:c>
       <x:c r="G103" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5037,7 +5037,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I103" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/431?comment=1130</x:v>
       </x:c>
       <x:c r="J103" s="6"/>
       <x:c r="K103" s="6" t="str">
@@ -5108,7 +5108,7 @@
         <x:v>К концу 2024 года в их списке есть и ЦСКА, и «Локомотив», и «Спартак», и «Динамо», иеще 267 других. «Торпедо» в их списке, кстати, нет. О чем речь?</x:v>
       </x:c>
       <x:c r="F105" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Станции Московского метрополитена</x:v>
       </x:c>
       <x:c r="G105" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5117,7 +5117,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I105" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/437?comment=1156</x:v>
       </x:c>
       <x:c r="J105" s="6"/>
       <x:c r="K105" s="6" t="str">
@@ -5148,7 +5148,7 @@
         <x:v>В ребрендинге 2020 года одной национальной команды на эмблеме объединили четырех мифических хранителей — быка, орла, дракона и великана; новый знак заменил прежний щит с аббревиатурой федерации и флагом. Согласно пресс-релизу, эти фигуры - традиционные защитники страны и мотив, связанный с государственной символикой. Назовите сборную, которая впервые добралась до ЧМ и ЧЕ лишь в ХХ! веке.</x:v>
       </x:c>
       <x:c r="F106" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Исландия</x:v>
       </x:c>
       <x:c r="G106" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5157,7 +5157,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I106" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/438?comment=1158</x:v>
       </x:c>
       <x:c r="J106" s="6"/>
       <x:c r="K106" s="6" t="str">
@@ -5188,7 +5188,7 @@
         <x:v>Шахматы 1922 года по модели Натальи Данько являются заметным образцом агитационного фарфора. В целях пропаганды скульптор придумала новые образы для каждой фигуры и заменила один из их традиционных цветов. Напишите пару цветов в версии шахмат Натальи Данько.</x:v>
       </x:c>
       <x:c r="F107" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Красные и белые</x:v>
       </x:c>
       <x:c r="G107" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5197,7 +5197,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I107" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/441?comment=1176</x:v>
       </x:c>
       <x:c r="J107" s="6"/>
       <x:c r="K107" s="6" t="str">
@@ -5268,7 +5268,7 @@
         <x:v>Около 10 лет назад у очень многих сильных игроков в фифу была определенная особенность в никнейме, поэтому их называли ИКСАМИ. Позднее термин трансформировался, и ИКСАМИ стали называть всех сильных игроков вне зависимости от того, какой у них никнейм. ИКСОМ можно назвать, например, Мохамеда Салаха, Рияда Мареза или Ашрафа Хакими. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F109" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Араб</x:v>
       </x:c>
       <x:c r="G109" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5277,7 +5277,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I109" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/450?comment=1196</x:v>
       </x:c>
       <x:c r="J109" s="6"/>
       <x:c r="K109" s="6" t="str">
@@ -5348,7 +5348,7 @@
         <x:v>В саундтреке FIFA 07 была песня этой группы. У этого трека 99 миллионов прослушиваний в Spotify, а у самой популярной песни группы - больше 2 миллиардов. Название этой группы совпадает с фамилиями двух легендарных игроков АПЛ. Один сыграл больше 200 матчей за «Тоттенхэм» и заезжал на сезон в «Ливерпуль». Другой провел больше 300 матчей за «МЮ». Как называется группа?</x:v>
       </x:c>
       <x:c r="F111" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Keane</x:v>
       </x:c>
       <x:c r="G111" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5357,7 +5357,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I111" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/452?comment=1215</x:v>
       </x:c>
       <x:c r="J111" s="6"/>
       <x:c r="K111" s="6" t="str">
@@ -5388,7 +5388,7 @@
         <x:v>До 2006 года там не фигурировал никто, а после 2022-го там можно было увидеть следующих исполнителей: Drake, The Rolling Stones, Coldplay, Karol С, Rosalia, Travis Scott. В этом списке могли быть Тэйлор Свифт и Эд Ширан, но пока не срослось. Что объединяет вышеуказанных артистов?</x:v>
       </x:c>
       <x:c r="F112" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Игровые футболки «Барселоны»</x:v>
       </x:c>
       <x:c r="G112" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5397,7 +5397,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I112" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/454?comment=1220</x:v>
       </x:c>
       <x:c r="J112" s="6"/>
       <x:c r="K112" s="6" t="str">
@@ -5428,7 +5428,7 @@
         <x:v>Дженнифер Лоуренс, Орландо Блум, Джереми Реннер, Рассел Кроу, Стивен Амелл - всех этих актеров объединяет некий олимпийский вид спорта. Назовите этот вид спорта.</x:v>
       </x:c>
       <x:c r="F113" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Стрельба из лука</x:v>
       </x:c>
       <x:c r="G113" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5437,7 +5437,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I113" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/467?comment=1262</x:v>
       </x:c>
       <x:c r="J113" s="6"/>
       <x:c r="K113" s="6" t="str">
@@ -5468,7 +5468,7 @@
         <x:v>Перед вами зашифрован персонаж культового произведения английского писателя. Мы уверены, что сам персонаж с легкостью прочел бы указанный SYXFRR EK Sete Однофамилец этого персонажа провел 10 сезонов в НБА. Он поиграл в «Филадельфии», «Финиксе», «Сакраменто», «Далласе» и «Вашингтоне». Он до сих пор в лиге. Назовите фамилию персонажа. Или баскетболиста.</x:v>
       </x:c>
       <x:c r="F114" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Шерлок Холмс</x:v>
       </x:c>
       <x:c r="G114" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5477,7 +5477,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I114" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/468?comment=1272</x:v>
       </x:c>
       <x:c r="J114" s="6"/>
       <x:c r="K114" s="6" t="str">
@@ -5508,7 +5508,7 @@
         <x:v>В США расфорсился скриншот с матча МЛБ между «Чикаго Кабс» и «Питтсбургом». На этом скриншоте видны упрощенные лого команд- участниц и счет матча, в котором одна из команд пока не набрала очков. Символы на этом скриншоте повторяют имя персонажа, фигурировавшего во всех эпизодах известнейшей франшизы. Напишите имя этого персонажа.</x:v>
       </x:c>
       <x:c r="F115" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>C-3PO</x:v>
       </x:c>
       <x:c r="G115" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5517,7 +5517,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I115" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/469?comment=1291</x:v>
       </x:c>
       <x:c r="J115" s="6"/>
       <x:c r="K115" s="6" t="str">
@@ -5548,7 +5548,7 @@
         <x:v>ИКС ИГРЕК - двукратный чемпион НБА, бронзовый призер Олимпийских игр и чемпион мира. ИКС ЗЕТ - звезда НФЛ, которая с 2019 года играет в одной команде. ИПСИЛОН ИКС - обладатель 22 наград «Грэмми». С НФЛ он так или иначе тоже связан. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F116" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Ламар</x:v>
       </x:c>
       <x:c r="G116" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5557,7 +5557,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I116" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/473?comment=1323</x:v>
       </x:c>
       <x:c r="J116" s="6"/>
       <x:c r="K116" s="6" t="str">
@@ -5588,7 +5588,7 @@
         <x:v>После поражения сборной Англии по крикету от Австралии в 1882 году The Sporting Times напечатали некролог: «Английский крикет умер 29 августа 1882 года». С тех пор победителям серии матчей между Англией и Австралией в тестовом крикете вручается ОНА. Возможно, если бы EE подарили вам, это вызвало быу вас как минимум непонимание, ау некоторых - даже обиду. Назовите EE двумя словами.</x:v>
       </x:c>
       <x:c r="F117" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Урна</x:v>
       </x:c>
       <x:c r="G117" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5597,7 +5597,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I117" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/474?comment=1332</x:v>
       </x:c>
       <x:c r="J117" s="6"/>
       <x:c r="K117" s="6" t="str">
@@ -5628,7 +5628,7 @@
         <x:v>Один из текстов на сайте Eurosport.ru, посвященный триумфу одной биатлонистки, был озаглавлен «ОНА маслом». ОНА - фамилия спортсменки, забравшейся на подиум. Назовите ЕЕ.</x:v>
       </x:c>
       <x:c r="F118" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Надежда Скардино</x:v>
       </x:c>
       <x:c r="G118" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5637,7 +5637,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I118" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/505?comment=1448</x:v>
       </x:c>
       <x:c r="J118" s="6"/>
       <x:c r="K118" s="6" t="str">
@@ -5668,7 +5668,7 @@
         <x:v>Перед вами список спортсменов: легкоатлет Ноа Лайлз, гольфист Брайсон Дешамбо, теннисистка Серена Уильямс, бейсболист Аарон Джадж, футболисты Неймар и Криштиану Роналду, баскетболисты Стефен Карри и Дэмиан Лиллард. В 2024 и 2025 гг. их медийно объединил один человек 1998 года рождения, чье настоящее имя — Джеймс Стивен Дональдсон. Назовите псевдоним этого человека.</x:v>
       </x:c>
       <x:c r="F119" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>MrBeast</x:v>
       </x:c>
       <x:c r="G119" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5677,7 +5677,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I119" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/507?comment=1459</x:v>
       </x:c>
       <x:c r="J119" s="6"/>
       <x:c r="K119" s="6" t="str">
@@ -5708,7 +5708,7 @@
         <x:v>Имена Диего Марадоны, Майка Тайсона, Роналдиньо, Флойда Мэйуэзера, Аллена Айверсона фигурировали в различных ИХ. В архитектуре ОН, помимо самых известных, бывает коринфским или тосканским. Назовите ЕГО.</x:v>
       </x:c>
       <x:c r="F120" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Ордер</x:v>
       </x:c>
       <x:c r="G120" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5717,7 +5717,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I120" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/508?comment=1461</x:v>
       </x:c>
       <x:c r="J120" s="6"/>
       <x:c r="K120" s="6" t="str">
@@ -5748,7 +5748,7 @@
         <x:v>Эта аббревиатура в какой-то степени ассоциируется с темнокожими людьми, правда, не в спортивных медиа, а в диджитал-файлах совершенно другого типа. A еще эта аббревиатура - название медиа, у которого есть не только спортивный раздел, но и целое пан- Африканское направление и редакция. Воспроизведите эту аббревиатуру, состоящую из трех латинских букв.</x:v>
       </x:c>
       <x:c r="F121" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>BBC</x:v>
       </x:c>
       <x:c r="G121" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5757,7 +5757,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I121" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/509?comment=1466</x:v>
       </x:c>
       <x:c r="J121" s="6"/>
       <x:c r="K121" s="6" t="str">
@@ -5788,7 +5788,7 @@
         <x:v>В романтическом плане Матвея Сафонова можно назвать ИМ - например, для его жены Марины. OH на французском языке — фамилия одного из партнеров Сафонова. Также ОН во Франции- низшая категория ордена Почетного легиона. Назовите ЕГО французским словом.</x:v>
       </x:c>
       <x:c r="F122" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Chevalier (шевалье)</x:v>
       </x:c>
       <x:c r="G122" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5797,7 +5797,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I122" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/511?comment=1483</x:v>
       </x:c>
       <x:c r="J122" s="6"/>
       <x:c r="K122" s="6" t="str">
@@ -5828,7 +5828,7 @@
         <x:v>В Северной Америке ТАК называют скамейки на матчах по бейсболу и американскому футболу, а также зрителей на этих играх. Одна из версий происхождения термина - что деревянные скамейки выгорали или выцветали на солнце. Также ЭТО СЛОВО присутствует в названии американского спортивного медиа, основанного в 2005 году. По сути, первые тексты создателей сайта стали взглядом с этих самых скамеек. Назовите слово или спортивное медиа.</x:v>
       </x:c>
       <x:c r="F123" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Bleachers</x:v>
       </x:c>
       <x:c r="G123" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5837,7 +5837,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I123" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/512?comment=1490</x:v>
       </x:c>
       <x:c r="J123" s="6"/>
       <x:c r="K123" s="6" t="str">
@@ -5868,7 +5868,7 @@
         <x:v>Если бы Артем Дзюба провел всю карьеру в «Спартаке», то из-за одного факта биографии форварда на «Лукойл Арене» его могли бы называть ИКСом. ИКС - прозвище заметного политического деятеля, который жил в России на стыке 16-го и Т7-го веков. Назовите ИКС двумя словами.</x:v>
       </x:c>
       <x:c r="F124" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тушинский вор</x:v>
       </x:c>
       <x:c r="G124" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5877,7 +5877,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I124" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/514?comment=1494</x:v>
       </x:c>
       <x:c r="J124" s="6"/>
       <x:c r="K124" s="6" t="str">
@@ -5908,7 +5908,7 @@
         <x:v>В топ-100 прямых эфиров на американском телевидении в 2023 году вошли сразу 97 спортивных трансляций. 94 из них - это матчи NFL. A 3 оставшихся?</x:v>
       </x:c>
       <x:c r="F125" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>NCAA</x:v>
       </x:c>
       <x:c r="G125" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5917,7 +5917,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I125" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/516?comment=1508</x:v>
       </x:c>
       <x:c r="J125" s="6"/>
       <x:c r="K125" s="6" t="str">
@@ -5948,7 +5948,7 @@
         <x:v>Карьера Сергея Юрьевича началась в клубе из Узбекистана в 1991 году, а завершилась в 2018 году в клубе из Белгорода. Сергей Юрьевич - олимпийский чемпион. Карьера Павла Сергеевича началась в 2017 году в клубе из Белгорода. Назовите фамилию Сергея Юрьевича и Павла Сергеевича.</x:v>
       </x:c>
       <x:c r="F126" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сергей Тетюхин</x:v>
       </x:c>
       <x:c r="G126" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5957,7 +5957,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I126" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/517?comment=1514</x:v>
       </x:c>
       <x:c r="J126" s="6"/>
       <x:c r="K126" s="6" t="str">
@@ -5988,7 +5988,7 @@
         <x:v>В 1999 году «Манчестер Сити» подписал контракт с издательством Eidos Interactive. С анонса того соглашения осталось несколько фотографий с НЕЙ. В 2020 году сайт Coop-Land признал EE грудь лучшей в истории индустрии. Кого мы загадали под НЕЙ?</x:v>
       </x:c>
       <x:c r="F127" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лара Крофт</x:v>
       </x:c>
       <x:c r="G127" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -5997,7 +5997,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I127" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/518?comment=1518</x:v>
       </x:c>
       <x:c r="J127" s="6"/>
       <x:c r="K127" s="6" t="str">
@@ -6028,7 +6028,7 @@
         <x:v>В одном из спешалов комик Эндрю Шульц рассуждал о разнице между Чикаго и Нью-Иорком. Он обратил внимание, что, в отличие от нью-йоркцев, жители Чикаго гордятся трагедиями в городе настолько, что даже назвали команду по футболу - «Чикаго Файр» -— якобы в честь великого чикагского пожара 1871 года. Когда Шульц начал рассуждать о названиях команд в Нью- Иорке, зал взорвался от смеха. Название какой команды вызвало у зрителей истерику?</x:v>
       </x:c>
       <x:c r="F128" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Jets</x:v>
       </x:c>
       <x:c r="G128" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6037,7 +6037,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I128" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/519?comment=1527</x:v>
       </x:c>
       <x:c r="J128" s="6"/>
       <x:c r="K128" s="6" t="str">
@@ -6068,7 +6068,7 @@
         <x:v>Блогер Софья Шамсутдинова ведет блог на «Спортсе”» и снимает рилзы Ha тему того, как учится играть в футбол: в роликах она чеканит мяч и делает разнообразные трюки. Название ее блога - каламбур, связанный сее именем и хорватским ресурсом, помогающим следить за ходом матча. Воспроизведите ее никнейм на «Спортсе”» и в других соцсетях.</x:v>
       </x:c>
       <x:c r="F129" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Sofascore</x:v>
       </x:c>
       <x:c r="G129" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6077,7 +6077,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I129" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/520?comment=1530</x:v>
       </x:c>
       <x:c r="J129" s="6"/>
       <x:c r="K129" s="6" t="str">
@@ -6148,7 +6148,7 @@
         <x:v>Фотограф Денис Тырин опубликовал фотографию с турнира по фигурному катанию. Благодаря талантливому кадрированию фото от названия турнира на рекламном щите за спиной Аделии Петросян осталось лишь шесть букв, что добавило фотографии дополнительный смысл. Эти шесть букв вы можете найти даже в первом абзаце вопроса. Напишите их.</x:v>
       </x:c>
       <x:c r="F131" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Пофигу</x:v>
       </x:c>
       <x:c r="G131" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6157,7 +6157,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I131" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/524?comment=1570</x:v>
       </x:c>
       <x:c r="J131" s="6"/>
       <x:c r="K131" s="6" t="str">
@@ -6188,7 +6188,7 @@
         <x:v>ИКС - фамилия довольно известного монстра. Если к ИКСУ добавить гласную букву и еще один орфографический знак, получится совершенно другой монстр: семикратный чемпион мира, выступающий на про-уровне вот уже 33 года. Назовите вид спорта, в котором выступает второй монстр.</x:v>
       </x:c>
       <x:c r="F132" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Снукер</x:v>
       </x:c>
       <x:c r="G132" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6197,7 +6197,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I132" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/527?comment=1578</x:v>
       </x:c>
       <x:c r="J132" s="6"/>
       <x:c r="K132" s="6" t="str">
@@ -6228,7 +6228,7 @@
         <x:v>Среди экс-комментаторов «НТВ-Плюс», оказавшихся на «Матч ТВ», пригласили и ЗАМЕНА. ЗАМЕНА - один из футболистов «Комо». Игрок проводит лишь первый сезон в Серии А после трансфера из загребского «Динамо». Что мы зашифровали под ЗАМЕНА?</x:v>
       </x:c>
       <x:c r="F133" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Батурина</x:v>
       </x:c>
       <x:c r="G133" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6237,7 +6237,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I133" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/535?comment=1607</x:v>
       </x:c>
       <x:c r="J133" s="6"/>
       <x:c r="K133" s="6" t="str">
@@ -6268,7 +6268,7 @@
         <x:v>В диджитал-версии журнала «Коммерсантъ» публикация, посвященная победе Андрея Рублева над Роджером Федерером, была озаглавлена следующим образом: «Андрей Рублев СДЕЛАЛ ЭТО». В 1904 году в Казанском Богородицком монастыре СДЕЛАЛИ ЭТО - это один из самых известных подобных случаев в России. Закончите заголовок «Коммерсанта» двумя словами.</x:v>
       </x:c>
       <x:c r="F134" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Вынес икону</x:v>
       </x:c>
       <x:c r="G134" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6277,7 +6277,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I134" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/542?comment=1619</x:v>
       </x:c>
       <x:c r="J134" s="6"/>
       <x:c r="K134" s="6" t="str">
@@ -6308,7 +6308,7 @@
         <x:v>Довольно известный русский иконописец ИКС родился и вырос в Византии, поэтому вошел в историю как ИКС ИГРЕК. Сразу 23 чемпиона Европы по футболу в 21-м веке были ИГРЕКАМИ. Назовите ИГРЕК.</x:v>
       </x:c>
       <x:c r="F135" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Феофан Грек</x:v>
       </x:c>
       <x:c r="G135" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6317,7 +6317,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I135" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/544?comment=1627</x:v>
       </x:c>
       <x:c r="J135" s="6"/>
       <x:c r="K135" s="6" t="str">
@@ -6348,7 +6348,7 @@
         <x:v>В средневековье во время осады города вражескими войсками в населенном пункте зачастую начинался ОН. Вы можете знать другого ЕГО: он периодически появляется в студии «Матч ТВ». Назовите ЕГО.</x:v>
       </x:c>
       <x:c r="F136" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мор</x:v>
       </x:c>
       <x:c r="G136" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6357,7 +6357,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I136" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/545?comment=1634</x:v>
       </x:c>
       <x:c r="J136" s="6"/>
       <x:c r="K136" s="6" t="str">
@@ -6388,7 +6388,7 @@
         <x:v>ИИ-художник jslayart составил несколько ростеров по определенному принципу. В одну команду вошли Джейлен Брансон, Наруто, Гоку, Существо, Микеланджело, Аанг. В другую - Патрик Махоумс, Майкл Джордан, Флеш, Тайгер Вудс, Дэдпул. В третью - Ламар Джексон, TaHoc, Джокер, Канг Завоеватель, Фриза. По какому принципу составлены эти ростеры?</x:v>
       </x:c>
       <x:c r="F137" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>По цветам костюмов: оранжевый, красный, фиолетовый</x:v>
       </x:c>
       <x:c r="G137" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6397,7 +6397,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I137" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/551?comment=1657</x:v>
       </x:c>
       <x:c r="J137" s="6"/>
       <x:c r="K137" s="6" t="str">
@@ -6428,7 +6428,7 @@
         <x:v>В январе 2013 года Ha Sports.ru вышел пост Кирилла Благова, посвященный лишнему весу звезды РПЛ из Эквадора. Вторая часть заголовка выглядела так: «Как отпуск Кайседо превратился в событие». Первая состояла из имени и фамилии известного южноамериканского спортсмена. Воспроизведите каламбур из первой части заголовка.</x:v>
       </x:c>
       <x:c r="F138" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Фелипе Масса</x:v>
       </x:c>
       <x:c r="G138" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6437,7 +6437,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I138" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/552?comment=1660</x:v>
       </x:c>
       <x:c r="J138" s="6"/>
       <x:c r="K138" s="6" t="str">
@@ -6468,7 +6468,7 @@
         <x:v>Серхио Перес, Сергей Карякин, Артур Шилов - всех их называли ИМ. Маурицио Сарри называл ИМ Лучано Спаллетти. Действующего ЕГО мы называть не будем. Назовите ЕГО двумя словами.</x:v>
       </x:c>
       <x:c r="F139" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Министр обороны</x:v>
       </x:c>
       <x:c r="G139" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6477,7 +6477,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I139" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/553?comment=1668</x:v>
       </x:c>
       <x:c r="J139" s="6"/>
       <x:c r="K139" s="6" t="str">
@@ -6508,7 +6508,7 @@
         <x:v>ОНО - один из самых популярных фильмов Брайана Де Пальмы. ОНО - прозвище культового футболиста, который отбегал 17 матчей за «Галатасарай», а потом 17 лет играл исключительно в клубах из топ-5 лиг Европы. Что такое ОНО? Ответьте тремя словами.</x:v>
       </x:c>
       <x:c r="F140" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лицо со шрамом</x:v>
       </x:c>
       <x:c r="G140" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6517,7 +6517,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I140" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/555?comment=1673</x:v>
       </x:c>
       <x:c r="J140" s="6"/>
       <x:c r="K140" s="6" t="str">
@@ -6548,7 +6548,7 @@
         <x:v>_—— ss В 2021 году в Германии выпустили 110 почтовые марки, посвященные 25- о к Fa С летнему юбилею победы ЕГО a АА. ag м4 *у над действующим на тот момент им а ем 3 тг AS dy Hye чемпионом мира Гарри Каспаровым. и мм “a ast i Несмотря на то, что мы скрыли 2 ЖЕ! фрагмент марки, вы все равно можете a F рассмотреть ЕГО на изображении. САВЕ! KASPAROW 20216 Назовите ЕГО имя двумя английскими словами абсолютно точно.</x:v>
       </x:c>
       <x:c r="F141" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Deep Blue</x:v>
       </x:c>
       <x:c r="G141" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6557,7 +6557,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I141" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/561?comment=1686</x:v>
       </x:c>
       <x:c r="J141" s="6"/>
       <x:c r="K141" s="6" t="str">
@@ -6588,7 +6588,7 @@
         <x:v>В США начали принимать ставки на то, кто СДЕЛАЕТ ЭТО до 2027 года. Иронично, что шансы на то, что Леброн Джеймс СДЕЛАЕТ ЭТО до 2027 года, оценивают выше, чем шансы на чемпионство «Лейкерс». Согласно котировкам букмекеров, шансы Леброна на то, что он СДЕЛАЕТ ЭТО до 2027 года, ниже, чем, например, владельца «Далласа» Марка Кьюбана, экс-игрока НФЛ Тома Брэйди, спортивного аналитика Стивена Эй Смита, а еще - Дуэйна «Скалы» Джонсона, Джорджа Клуни, Илона Маска и Ким Кардашьян. Что мы зашифровали под СДЕЛАЕТ ЭТО?</x:v>
       </x:c>
       <x:c r="F142" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Объявит о выдвижении в президенты</x:v>
       </x:c>
       <x:c r="G142" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6597,7 +6597,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I142" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/567?comment=1698</x:v>
       </x:c>
       <x:c r="J142" s="6"/>
       <x:c r="K142" s="6" t="str">
@@ -6628,7 +6628,7 @@
         <x:v>В 1921 году британец Гарольд Сирлс Торнтон запатентовал некое устройство. Его структуру можно описать числовым рядом «123553 2 I». Сейчас многие из вас знают это устройство как ИКС Другой ИКС, который вы тоже можете знать, был основан на год раньше, в 1920 году в Нюрнберге. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F143" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кикер</x:v>
       </x:c>
       <x:c r="G143" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6637,7 +6637,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I143" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/568?comment=1706</x:v>
       </x:c>
       <x:c r="J143" s="6"/>
       <x:c r="K143" s="6" t="str">
@@ -6668,7 +6668,7 @@
         <x:v>В 2008 году сайт Goal.com опубликовал пост, посвященный поражению «Ювентуса» в еврокубковом матче. Он звучал на английском так: «Old Lady unable to master ПРОПУСК at home». Разумеется, в заголовке зашифрована игра слов, причем довольно непристойная. Заполните ПРОПУСК четырьмя буквами.</x:v>
       </x:c>
       <x:c r="F144" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>БАТЭ</x:v>
       </x:c>
       <x:c r="G144" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6677,7 +6677,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I144" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/569?comment=1709</x:v>
       </x:c>
       <x:c r="J144" s="6"/>
       <x:c r="K144" s="6" t="str">
@@ -6708,7 +6708,7 @@
         <x:v>«Википедия» считает, что одна ОНА больше известна под фамилией Белобородова. МОК аннулировал ее золотую медаль Олимпиады-2012. Другая ОНА имела непосредственное отношение к интеллектуальным играм, но стала известной благодаря спортивным медиа. ОН - один из самых заметных и известных журналистов «Чемпионата». Какая фамилия объединяет этих людей?</x:v>
       </x:c>
       <x:c r="F145" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лысенко</x:v>
       </x:c>
       <x:c r="G145" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6717,7 +6717,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I145" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/570?comment=1715</x:v>
       </x:c>
       <x:c r="J145" s="6"/>
       <x:c r="K145" s="6" t="str">
@@ -6788,7 +6788,7 @@
         <x:v>50 Cent - 21 ИКС. Обладатель второго места конкурса комментаторов «России-2» в 2012 году - 50 ИКСОВ. Чему равен ИКС?</x:v>
       </x:c>
       <x:c r="F147" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Вопрос (question)</x:v>
       </x:c>
       <x:c r="G147" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6797,7 +6797,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I147" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/572?comment=1728</x:v>
       </x:c>
       <x:c r="J147" s="6"/>
       <x:c r="K147" s="6" t="str">
@@ -6828,7 +6828,7 @@
         <x:v>В пьесе «Двенадцатая ночь» Уильям Шекспир писал, что дурацкий колпак ПРОПУСК не портит. ПРОПУСК точно не испортил «Кливленд» в 2016 году, ведь команда стала чемпионом НБА. Восполните ПРОПУСК.</x:v>
       </x:c>
       <x:c r="F148" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мозгов</x:v>
       </x:c>
       <x:c r="G148" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6837,7 +6837,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I148" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/587?comment=1781</x:v>
       </x:c>
       <x:c r="J148" s="6"/>
       <x:c r="K148" s="6" t="str">
@@ -6868,7 +6868,7 @@
         <x:v>Матч «Арсенала» и «Кристал Пэласа» 1 января 2017 года вызвал много шуток и реакций в соцсетях и на спортивных сайтах из-за ЕГО гола: русскоязычные фанаты футбола посчитали ЕГО гол довольно символичным. Кто забил гол в том матче?</x:v>
       </x:c>
       <x:c r="F149" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Оливье Жиру</x:v>
       </x:c>
       <x:c r="G149" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6877,7 +6877,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I149" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/588?comment=1793</x:v>
       </x:c>
       <x:c r="J149" s="6"/>
       <x:c r="K149" s="6" t="str">
@@ -6908,7 +6908,7 @@
         <x:v>ОН на английском - бывший футболист, забивавший за «Лацио» и «Рейнджерс». ОН на русском - главный герой мультфильма «Пес в сапогах». Назовите ЕГО по-английски или по-русски.</x:v>
       </x:c>
       <x:c r="F150" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Gascoigne / Гасконец</x:v>
       </x:c>
       <x:c r="G150" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6917,7 +6917,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I150" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/589?comment=1796</x:v>
       </x:c>
       <x:c r="J150" s="6"/>
       <x:c r="K150" s="6" t="str">
@@ -6948,7 +6948,7 @@
         <x:v>Жительница Манилы четыре года молилась статуэтке ИКСА, ошибочно думая, что это Хотэй - популярное в китайской культуре божество счастья, благополучия, веселья и общения. Ее смутил большой живот статуэтки. ИКС — прозвище футболиста, который по завершении карьеры потренировал клубы из Вашингтона, Плимута, Бирмингема и Дерби. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="F151" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Шрек</x:v>
       </x:c>
       <x:c r="G151" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6957,7 +6957,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I151" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/594?comment=1806</x:v>
       </x:c>
       <x:c r="J151" s="6"/>
       <x:c r="K151" s="6" t="str">
@@ -6988,7 +6988,7 @@
         <x:v>На альбоме «Пиры и раны» группы «Кровосток» есть песна «ЗАМЕНА». ЗАМЕНА состоит из двух глаголов, которые образуют фразу, используемую для ироничного описания тактики некоторых футбольных команд. ЗАМЕНА - правда, с чуть измененной орфографией, — название ныне несуществующей медиафутбольной команды. Воспроизведите ЗАМЕНУ.</x:v>
       </x:c>
       <x:c r="F152" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Бей-беги</x:v>
       </x:c>
       <x:c r="G152" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -6997,7 +6997,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I152" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/601?comment=1828</x:v>
       </x:c>
       <x:c r="J152" s="6"/>
       <x:c r="K152" s="6" t="str">
@@ -7028,7 +7028,7 @@
         <x:v>Сайт 9meters подсчитал, что в мире живет 2700 ТАКИХ людей. 33 из 2700 ТАКИХ людей играют в НБА. ТАКИЕ - составное прилагательное, причем второй корень очень редко используется в России и часто — в США. Что мы зашифровали под ТАКИМИ?</x:v>
       </x:c>
       <x:c r="F153" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Семифутеры</x:v>
       </x:c>
       <x:c r="G153" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7037,7 +7037,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I153" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/604?comment=1835</x:v>
       </x:c>
       <x:c r="J153" s="6"/>
       <x:c r="K153" s="6" t="str">
@@ -7068,7 +7068,7 @@
         <x:v>АЛЬФОЙ в славянской мифологии называли духа умершего человека в облике женщины. Известная вам АЛЬФА - олимпийская чемпионка, которая сначала вышла замуж за тренера, а затем — за человека, в честь отличительной особенности которого назвали либеральное микромедиа. Назовите АЛЬФУ.</x:v>
       </x:c>
       <x:c r="F154" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Навка</x:v>
       </x:c>
       <x:c r="G154" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7077,7 +7077,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I154" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/607?comment=1843</x:v>
       </x:c>
       <x:c r="J154" s="6"/>
       <x:c r="K154" s="6" t="str">
@@ -7108,7 +7108,7 @@
         <x:v>Поговорим о маршрутах. Из «Селтикс» в «Суперсоникс» - 90. Из «Селтикс» в «Уорриорз» - 80. Из «Уизардс» в «Уорриорз» - 50. Число, которое соответствует маршруту Пау Газоля в 2014-м, вы прекрасно знаете: ему посвящено много отсылок в поп-культуре. Назовите его.</x:v>
       </x:c>
       <x:c r="F155" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Route 66</x:v>
       </x:c>
       <x:c r="G155" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7117,7 +7117,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I155" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/611?comment=1858</x:v>
       </x:c>
       <x:c r="J155" s="6"/>
       <x:c r="K155" s="6" t="str">
@@ -7148,7 +7148,7 @@
         <x:v>Если бы популярный российский блогер получил прозвище, потому что он EE сын, это было бы намного более логично. Но нет: несмотря на совпадение фамилий, он не состоит с НЕЙ в родственных связях. ОНА завоевала серебряную медаль на ОИ в Сиднее и сразу две медали - золото и бронзу - в Афинах. Назовите EE имя и фамилию.</x:v>
       </x:c>
       <x:c r="F156" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Татьяна Лебедева</x:v>
       </x:c>
       <x:c r="G156" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7157,7 +7157,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I156" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/613?comment=1860</x:v>
       </x:c>
       <x:c r="J156" s="6"/>
       <x:c r="K156" s="6" t="str">
@@ -7188,7 +7188,7 @@
         <x:v>Один ОН - французский автогонщик, девятикратный чемпион мира. Другой ОН - немецкий автогонщик, четырехкратный чемпион мира. Было бы символично, если бы и первый, и второй ОН одержали победы в одном испанском городе, но гонки, в которых они принимали участие, в нем не проходили. Назовите ЕГО.</x:v>
       </x:c>
       <x:c r="F157" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сан-Себастьян</x:v>
       </x:c>
       <x:c r="G157" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7197,7 +7197,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I157" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/617?comment=1870</x:v>
       </x:c>
       <x:c r="J157" s="6"/>
       <x:c r="K157" s="6" t="str">
@@ -7228,7 +7228,7 @@
         <x:v>1988, 1992, 1996, 2000 - ПЕРВЫЕ. 1988, 1992, 1994, 1998 —- ВТОРЫЕ. Назовите ПЕРВЫЕ и ВТОРЫЕ.</x:v>
       </x:c>
       <x:c r="F158" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Летние и зимние Олимпийские игры</x:v>
       </x:c>
       <x:c r="G158" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7237,7 +7237,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I158" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/618?comment=1874</x:v>
       </x:c>
       <x:c r="J158" s="6"/>
       <x:c r="K158" s="6" t="str">
@@ -7268,7 +7268,7 @@
         <x:v>«Манчестер Сити», «Интер», «Лилль», «Бавария», «Атлетико» - все эти клубы объединяет трек FRIENDLY THUG 52 МСС с альбома «Graf Monte-Cristo/Most Valuable Pirate». Воспроизведите название этого трека.</x:v>
       </x:c>
       <x:c r="F159" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="G159" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7277,7 +7277,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I159" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/620?comment=1884</x:v>
       </x:c>
       <x:c r="J159" s="6"/>
       <x:c r="K159" s="6" t="str">
@@ -7308,7 +7308,7 @@
         <x:v>В интернете можно найти победителей ЭТОГО турнира с 1949 года. Вот некоторые из них. 2025 - Джексон Шторм. 2024 - Пол Корнев. 2023 - Райан Лэйни. 2022 - Тим Тредлесс. 2021 - Круз Рамирес. 2020 - Чейз Рейселотт. В 2006, 2007, 2009, 2010, 2011, 2012 и 2015 годах победителем становился рекордсмен, которому даже посвятили серию фильмов. Назовите турнир, о котором идет речь.</x:v>
       </x:c>
       <x:c r="F160" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кубок Поршня</x:v>
       </x:c>
       <x:c r="G160" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7317,7 +7317,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I160" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/623?comment=1890</x:v>
       </x:c>
       <x:c r="J160" s="6"/>
       <x:c r="K160" s="6" t="str">
@@ -7348,7 +7348,7 @@
         <x:v>В английском языке для того, чтобы превратить фамилию главного героя культового сериала в фамилию члена Зала славы снукера, необходимо убрать согласную букву. В русском языке для того, чтобы превратить фамилию главного героя культового сериала в фамилию члена Зала славы снукера, необходимо заменить согласную букву. Назовите члена Зала славы снукера, о котором идет речь.</x:v>
       </x:c>
       <x:c r="F161" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Марк Селби</x:v>
       </x:c>
       <x:c r="G161" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7357,7 +7357,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I161" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/624?comment=1896</x:v>
       </x:c>
       <x:c r="J161" s="6"/>
       <x:c r="K161" s="6" t="str">
@@ -7388,7 +7388,7 @@
         <x:v>Обидно, что в «Орландо» нет футболиста по имени и фамилии Эйбел - они бы составили потрясающую, чуть ли не братскую связку с другим игроком «Мэджик». Назовите фамилию этого игрока - или ее русскоязычный аналог.</x:v>
       </x:c>
       <x:c r="F162" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Каин</x:v>
       </x:c>
       <x:c r="G162" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7397,7 +7397,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I162" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/625?comment=1898</x:v>
       </x:c>
       <x:c r="J162" s="6"/>
       <x:c r="K162" s="6" t="str">
@@ -7428,7 +7428,7 @@
         <x:v>Баскетболист «Никс» Карл-Энтони Таунс приехал на Матч звезд НБА в бомбере, на спине которого был изображен христианский святой в узнаваемом образе. Согласно житию этого святого, он родился в Каппадокии. А его изображение вы точно видели много раз. Возможно, вам помогут догадаться, где оно вам встречалось, числа 1, 5, 10 и 50. Назовите этого святого двумя словами.</x:v>
       </x:c>
       <x:c r="F163" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Георгий Победоносец</x:v>
       </x:c>
       <x:c r="G163" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7437,7 +7437,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I163" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/628?comment=1908</x:v>
       </x:c>
       <x:c r="J163" s="6"/>
       <x:c r="K163" s="6" t="str">
@@ -7468,7 +7468,7 @@
         <x:v>В 2021 году Леонид Слуцкий сделал ЕЕ: он рассказал об этом Ксении Собчак на ее УочТиБе-канале. С 2022 года многие россияне начали намного чаще делать EE, если хотят посетить страны Европы, Азии и Америки. Назовите EE тремя словами.</x:v>
       </x:c>
       <x:c r="F164" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Пересадка в Турции</x:v>
       </x:c>
       <x:c r="G164" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7477,7 +7477,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I164" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/664?comment=1977</x:v>
       </x:c>
       <x:c r="J164" s="6"/>
       <x:c r="K164" s="6" t="str">
@@ -7508,7 +7508,7 @@
         <x:v>Один из экспертов по русскому футболу дал такую характеристику 20-летнему форварду «Уфы» и воспитаннику одного из топ-клубов РПЛ Алексею Барановскому: «Он наглый пацан, который хорошо умеет играть в футбол. Говорю ему: все отлично, кроме фамилии». Назовите эксперта, который дал эту характеристику.</x:v>
       </x:c>
       <x:c r="F165" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Андрей Аршавин</x:v>
       </x:c>
       <x:c r="G165" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7517,7 +7517,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I165" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/669?comment=2000</x:v>
       </x:c>
       <x:c r="J165" s="6"/>
       <x:c r="K165" s="6" t="str">
@@ -7548,7 +7548,7 @@
         <x:v>Перед вами фрагмент постера, со Ма та посвященного одному =. м. ее спортивному событию. Горы, rh. которые стали частью Ч 4 а композиции, мы скрыли. AS ; Мы He спрашиваем вас, что А . это за событие - напишите, в 12 форме чего выполнен силуэт Ni города на этом постере. (5 R E</x:v>
       </x:c>
       <x:c r="F166" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Олимпийский факел</x:v>
       </x:c>
       <x:c r="G166" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7557,7 +7557,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I166" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/682?comment=2023</x:v>
       </x:c>
       <x:c r="J166" s="6"/>
       <x:c r="K166" s="6" t="str">
@@ -7588,7 +7588,7 @@
         <x:v>Обратная ОНА была распространенным приемом в византийской и древнерусской иконописи. Когда речь идет о талантливых спортсменах, часто говорят о НЕЙ и называют ТАКИМИ - прилагательным, образованным от слова ОНА. Правда, чем старше спортсмен, тем реже мы говорим о том, что он - ТАКОЙ. Даи ИХ у него становится меньше. Назовите EE.</x:v>
       </x:c>
       <x:c r="F167" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Перспектива</x:v>
       </x:c>
       <x:c r="G167" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7597,7 +7597,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I167" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/684?comment=2026</x:v>
       </x:c>
       <x:c r="J167" s="6"/>
       <x:c r="K167" s="6" t="str">
@@ -7668,7 +7668,7 @@
         <x:v>Несмотря на то, что эта европейская страна не попала на чемпионат мира по футболу, ее англоязычное название можно было увидеть во время трансляций как минимум восьми матчей ЧМ-2026. Назовите эту европейскую страну.</x:v>
       </x:c>
       <x:c r="F169" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Грузия</x:v>
       </x:c>
       <x:c r="G169" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7677,7 +7677,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I169" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/717?comment=2103</x:v>
       </x:c>
       <x:c r="J169" s="6"/>
       <x:c r="K169" s="6" t="str">
@@ -7708,7 +7708,7 @@
         <x:v>В 2006 году на платформе PSP вышла игра, где основной механикой был наклон планеты. Первая часть названия - испанское слово, которое совпадает с прозвищем тренера, не вышедшего вместе со сборной из группы на ЧМ-2026. Назовите фамилию этого тренера.</x:v>
       </x:c>
       <x:c r="F170" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Марсело Бьельса</x:v>
       </x:c>
       <x:c r="G170" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -7717,7 +7717,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I170" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ подтверждён реакцией канала: https://t.me/simple_quiz/718?comment=2108</x:v>
       </x:c>
       <x:c r="J170" s="6"/>
       <x:c r="K170" s="6" t="str">
@@ -7791,7 +7791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc1d16ff2fa64844"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4777c06e4b5047c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8467,7 +8467,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903b6a0acc924a33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefd9b9808a541f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8639,7 +8639,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e057e77005c45ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6631473d2eb847c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8903,7 +8903,7 @@
     <x:mergeCell ref="E9:H9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fcdbfcd6fee46ba"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58654fc5740548a6"/>
 </x:worksheet>
 </file>
 
@@ -9394,7 +9394,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4ffe42de32e4d68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb22a28fec224528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9431,7 +9431,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="44" t="str">
-        <x:v>130 распознанных карточек; 122 новых вопросов добавлено в «Каталог», 8 совпадений отмечено как дубликаты. Ответы отсутствуют на исходных карточках.</x:v>
+        <x:v>130 распознанных карточек; 122 новых вопросов добавлено в «Каталог», 8 совпадений отмечено как дубликаты. 113 ответов заполнено.</x:v>
       </x:c>
       <x:c r="B2" s="44"/>
       <x:c r="C2" s="44"/>
@@ -9475,7 +9475,7 @@
         <x:v>Дубликат ID</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="46" customHeight="1">
+    <x:row r="4" ht="72" customHeight="1">
       <x:c r="A4" s="48" t="str">
         <x:v>TG-0006</x:v>
       </x:c>
@@ -9489,7 +9489,7 @@
         <x:v>Этот сезон НХЛ - уникальный: домашний матч «Каролины» против «Тампа-Бэй» перенесли из-за НЕГО, а матч «Лос-Анджелеса» против «Калгари» перенесли из-за НИХ. Как иронично. Назовите ЕГО и ИХ.</x:v>
       </x:c>
       <x:c r="E4" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Ураган и пожары</x:v>
       </x:c>
       <x:c r="F4" s="50" t="str">
         <x:v>https://t.me/simple_quiz/6</x:v>
@@ -9501,11 +9501,11 @@
         <x:v>0.9424</x:v>
       </x:c>
       <x:c r="I4" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J4" s="48"/>
     </x:row>
-    <x:row r="5" ht="46" customHeight="1">
+    <x:row r="5" ht="72" customHeight="1">
       <x:c r="A5" s="48" t="str">
         <x:v>TG-0007</x:v>
       </x:c>
@@ -9519,7 +9519,7 @@
         <x:v>Если ты любитель спорта, то в Америке тебе не удастся сходить на рэп, поп или фолк, зато можно сходить на рок, на ИКС и на ИГРЕК. Назовите ИКС и ИГРЕК. о</x:v>
       </x:c>
       <x:c r="E5" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>«Юта Джаз» и «Сент-Луис Блюз»</x:v>
       </x:c>
       <x:c r="F5" s="50" t="str">
         <x:v>https://t.me/simple_quiz/7</x:v>
@@ -9531,11 +9531,11 @@
         <x:v>0.9414</x:v>
       </x:c>
       <x:c r="I5" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J5" s="48"/>
     </x:row>
-    <x:row r="6" ht="46" customHeight="1">
+    <x:row r="6" ht="72" customHeight="1">
       <x:c r="A6" s="48" t="str">
         <x:v>TG-0017</x:v>
       </x:c>
@@ -9549,7 +9549,7 @@
         <x:v>Рядом с ЭТИМ на футбольных матчах с 2020 года красуется цифра 5, с 2013 года - 4, с 2006 года - 3, с 2000 года - 2. А вообще ЭТО фигурирует в трансляциях некоторых футбольных матчей с 1995 года. О чем речь?</x:v>
       </x:c>
       <x:c r="E6" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>PS (PlayStation)</x:v>
       </x:c>
       <x:c r="F6" s="50" t="str">
         <x:v>https://t.me/simple_quiz/17</x:v>
@@ -9561,11 +9561,11 @@
         <x:v>0.9459</x:v>
       </x:c>
       <x:c r="I6" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J6" s="48"/>
     </x:row>
-    <x:row r="7" ht="46" customHeight="1">
+    <x:row r="7" ht="72" customHeight="1">
       <x:c r="A7" s="48" t="str">
         <x:v>TG-0019</x:v>
       </x:c>
@@ -9579,7 +9579,7 @@
         <x:v>Первая ОНА появились в России в 2001 году. Сейчас ИХ более 40 в Москве и Московской области. Ав 2018 году благодаря паре русских футболистов одна из НИХ на протяжении нескольких месяцев регулярно появлялась в новостных каналах и пабликах. Назовите EE.</x:v>
       </x:c>
       <x:c r="E7" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кофемания</x:v>
       </x:c>
       <x:c r="F7" s="50" t="str">
         <x:v>https://t.me/simple_quiz/19</x:v>
@@ -9591,11 +9591,11 @@
         <x:v>0.9548</x:v>
       </x:c>
       <x:c r="I7" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J7" s="48"/>
     </x:row>
-    <x:row r="8" ht="46" customHeight="1">
+    <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="48" t="str">
         <x:v>TG-0035</x:v>
       </x:c>
@@ -9625,7 +9625,7 @@
       </x:c>
       <x:c r="J8" s="48"/>
     </x:row>
-    <x:row r="9" ht="46" customHeight="1">
+    <x:row r="9" ht="72" customHeight="1">
       <x:c r="A9" s="48" t="str">
         <x:v>TG-0050</x:v>
       </x:c>
@@ -9655,7 +9655,7 @@
       </x:c>
       <x:c r="J9" s="48"/>
     </x:row>
-    <x:row r="10" ht="46" customHeight="1">
+    <x:row r="10" ht="72" customHeight="1">
       <x:c r="A10" s="48" t="str">
         <x:v>TG-0127</x:v>
       </x:c>
@@ -9669,7 +9669,7 @@
         <x:v>В 2014 году 21-летняя испанка Гарбинье Мугуруса сенсационно выбила из сетки «Ролан Гаррос» Серену Уильямс и добралась до до четвертьфинала турнира «Большого шлема». На сайте Eurosport.ru вышел пост с фактами про Гарбинье. Назывался он так: «Мугуруса, ПРОПУСК». Заголовок - аллюзия на популярную в середине 20 века фразу: она не раз звучала в самом известном фильме про пионеров. Какие два слова мы пропустили в заголовке текста на Eurosport.ru?</x:v>
       </x:c>
       <x:c r="E10" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>А что вы тут делаете, а?</x:v>
       </x:c>
       <x:c r="F10" s="50" t="str">
         <x:v>https://t.me/simple_quiz/127</x:v>
@@ -9681,11 +9681,11 @@
         <x:v>0.9424</x:v>
       </x:c>
       <x:c r="I10" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J10" s="48"/>
     </x:row>
-    <x:row r="11" ht="46" customHeight="1">
+    <x:row r="11" ht="72" customHeight="1">
       <x:c r="A11" s="48" t="str">
         <x:v>TG-0130</x:v>
       </x:c>
@@ -9699,7 +9699,7 @@
         <x:v>Было бы символично, если бы ИКС ИГРЕК играл за ЗЕТ ИКС, но нет: в США он выступал лишь за одну команду. Назовите ИКС. Если вы знаете, что за песня Queen играла в рекламе Coca-Cola, вам, скорее всего, будет проще справиться с этим вопросом.</x:v>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мэджик</x:v>
       </x:c>
       <x:c r="F11" s="50" t="str">
         <x:v>https://t.me/simple_quiz/130</x:v>
@@ -9711,11 +9711,11 @@
         <x:v>0.9566</x:v>
       </x:c>
       <x:c r="I11" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J11" s="48"/>
     </x:row>
-    <x:row r="12" ht="46" customHeight="1">
+    <x:row r="12" ht="72" customHeight="1">
       <x:c r="A12" s="48" t="str">
         <x:v>TG-0141</x:v>
       </x:c>
@@ -9729,7 +9729,7 @@
         <x:v>ЭТО есть как минимум в двух экземплярах у каждого профессионального клуба. ЭТО было и в названии одного из клубов НБА, нос 2012 года не фигурирует в нем. О чем речь?</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Джерси</x:v>
       </x:c>
       <x:c r="F12" s="50" t="str">
         <x:v>https://t.me/simple_quiz/141</x:v>
@@ -9741,11 +9741,11 @@
         <x:v>0.9559</x:v>
       </x:c>
       <x:c r="I12" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J12" s="48"/>
     </x:row>
-    <x:row r="13" ht="46" customHeight="1">
+    <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="48" t="str">
         <x:v>TG-0142</x:v>
       </x:c>
@@ -9759,7 +9759,7 @@
         <x:v>Назовите команду МФЛ, которая всегда располагается в таблице на 22-м месте.</x:v>
       </x:c>
       <x:c r="E13" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Титан</x:v>
       </x:c>
       <x:c r="F13" s="50" t="str">
         <x:v>https://t.me/simple_quiz/142</x:v>
@@ -9771,11 +9771,11 @@
         <x:v>0.9526</x:v>
       </x:c>
       <x:c r="I13" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J13" s="48"/>
     </x:row>
-    <x:row r="14" ht="46" customHeight="1">
+    <x:row r="14" ht="72" customHeight="1">
       <x:c r="A14" s="48" t="str">
         <x:v>TG-0145</x:v>
       </x:c>
@@ -9805,7 +9805,7 @@
       </x:c>
       <x:c r="J14" s="48"/>
     </x:row>
-    <x:row r="15" ht="46" customHeight="1">
+    <x:row r="15" ht="72" customHeight="1">
       <x:c r="A15" s="48" t="str">
         <x:v>TG-0157</x:v>
       </x:c>
@@ -9819,7 +9819,7 @@
         <x:v>Этот оскорбительный термин применительно к девушкам регулярно вспоминают в русскоязычном твиттере. В одном из олимпийских видов спорта так можно безоценочно назвать его представительниц. Среди олимпийских чемпионок в этом виде спорта в 21 веке - чилийка Франсиска Кроветто, американки Эмбер Инглиш и Ким Роуд, итальянки Диана Бакози и Кьяра Кайнеро, венгерка Диана Игали. Наверное, несправедливо, что некоторым из вас официанты принесли подсказку. Назовите этот термин.</x:v>
       </x:c>
       <x:c r="E15" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тарелочница</x:v>
       </x:c>
       <x:c r="F15" s="50" t="str">
         <x:v>https://t.me/simple_quiz/157</x:v>
@@ -9831,11 +9831,11 @@
         <x:v>0.9494</x:v>
       </x:c>
       <x:c r="I15" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J15" s="48"/>
     </x:row>
-    <x:row r="16" ht="46" customHeight="1">
+    <x:row r="16" ht="72" customHeight="1">
       <x:c r="A16" s="48" t="str">
         <x:v>TG-0178</x:v>
       </x:c>
@@ -9849,7 +9849,7 @@
         <x:v>Валентин Серов посвятил краже ИКС не одно полотно: говорят, он написал шесть вариантов картины. Карло Анчелотти вызвал 25 футболистов на первые для него у руля матчи сборной Бразилии. Четыре из них никогда не играли в ИКС. Несмотря на то, что технически вы в ИКС прямо сейчас, некоторые из вас могут похвастаться, что были в ИКС. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E16" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Европа</x:v>
       </x:c>
       <x:c r="F16" s="50" t="str">
         <x:v>https://t.me/simple_quiz/178</x:v>
@@ -9861,11 +9861,11 @@
         <x:v>0.9628</x:v>
       </x:c>
       <x:c r="I16" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J16" s="48"/>
     </x:row>
-    <x:row r="17" ht="46" customHeight="1">
+    <x:row r="17" ht="72" customHeight="1">
       <x:c r="A17" s="48" t="str">
         <x:v>TG-0180</x:v>
       </x:c>
@@ -9879,7 +9879,7 @@
         <x:v>В конце 15 века итальянский художник написал картину, на которой было изображено первое событие в жизни АЛЬФЫ. Картина была написана по заказу представителя семьи Медичи. Полотно до сих пор хранится в галерее Уффици. 17 июня 1980 года произошло первое событие в жизни другой АЛЬФЫ. Напишите в ответе название картины.</x:v>
       </x:c>
       <x:c r="E17" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>«Рождение Венеры»</x:v>
       </x:c>
       <x:c r="F17" s="50" t="str">
         <x:v>https://t.me/simple_quiz/180</x:v>
@@ -9891,11 +9891,11 @@
         <x:v>0.9617</x:v>
       </x:c>
       <x:c r="I17" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J17" s="48"/>
     </x:row>
-    <x:row r="18" ht="46" customHeight="1">
+    <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="48" t="str">
         <x:v>TG-0181</x:v>
       </x:c>
@@ -9909,7 +9909,7 @@
         <x:v>В английском языке это слово означает близкого друга, братишку. Если это же слово написать кириллицей, получится некое действие во множественном числе, свидетелем которого можно стать, например, в петанке, дартсе и водном поло. Напишите это слово кириллицей.</x:v>
       </x:c>
       <x:c r="E18" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Броски</x:v>
       </x:c>
       <x:c r="F18" s="50" t="str">
         <x:v>https://t.me/simple_quiz/181</x:v>
@@ -9921,11 +9921,11 @@
         <x:v>0.9583</x:v>
       </x:c>
       <x:c r="I18" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J18" s="48"/>
     </x:row>
-    <x:row r="19" ht="46" customHeight="1">
+    <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="48" t="str">
         <x:v>TG-0187</x:v>
       </x:c>
@@ -9939,7 +9939,7 @@
         <x:v>У группы Oasis и рэпера Big Baby Tape есть треки с одинаковым названием. Увидев название этих треков, в голову сразу приходит важный для истории НБА город. О каком городе речь?</x:v>
       </x:c>
       <x:c r="E19" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сиэтл</x:v>
       </x:c>
       <x:c r="F19" s="50" t="str">
         <x:v>https://t.me/simple_quiz/187</x:v>
@@ -9951,11 +9951,11 @@
         <x:v>0.9603</x:v>
       </x:c>
       <x:c r="I19" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J19" s="48"/>
     </x:row>
-    <x:row r="20" ht="46" customHeight="1">
+    <x:row r="20" ht="72" customHeight="1">
       <x:c r="A20" s="48" t="str">
         <x:v>TG-0206</x:v>
       </x:c>
@@ -9969,7 +9969,7 @@
         <x:v>Российского предпринимателя из Троицка, который открыл бизнес в Сыктывкаре, и линию обороны футбольного клуба «Рома» с 2012 по 2014. год, объединяют два повторяющихся слога. Напишите эти два одинаковых слога.</x:v>
       </x:c>
       <x:c r="E20" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Додо</x:v>
       </x:c>
       <x:c r="F20" s="50" t="str">
         <x:v>https://t.me/simple_quiz/206</x:v>
@@ -9981,11 +9981,11 @@
         <x:v>0.954</x:v>
       </x:c>
       <x:c r="I20" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J20" s="48"/>
     </x:row>
-    <x:row r="21" ht="46" customHeight="1">
+    <x:row r="21" ht="72" customHeight="1">
       <x:c r="A21" s="48" t="str">
         <x:v>TG-0207</x:v>
       </x:c>
@@ -10015,7 +10015,7 @@
       </x:c>
       <x:c r="J21" s="48"/>
     </x:row>
-    <x:row r="22" ht="46" customHeight="1">
+    <x:row r="22" ht="72" customHeight="1">
       <x:c r="A22" s="48" t="str">
         <x:v>TG-0213</x:v>
       </x:c>
@@ -10029,7 +10029,7 @@
         <x:v>В 2019 году в сторисах Sports.ru провели небольшой квиз из трех картинок. На первой была показана картина «Впечатление». Вопрос на картинке был следующим: «Это шедевр ИКСА?» Правильный ответ, конечно, — «Нет». На второй тот же вопрос с тем же ответом дали рядом с картиной «Олимпия». На третьей была фотография из матча «Ливерпуль» - «Бавария». Вопрос на картинке совпадал: «Это шедевр ИКСА?» Правильный ответ - «Да!» В ЛЧ-2018/19 ИКС забил 4 гола. Назовите ИКС двумя словами.</x:v>
       </x:c>
       <x:c r="E22" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Садио Мане</x:v>
       </x:c>
       <x:c r="F22" s="50" t="str">
         <x:v>https://t.me/simple_quiz/213</x:v>
@@ -10041,11 +10041,11 @@
         <x:v>0.9468</x:v>
       </x:c>
       <x:c r="I22" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J22" s="48"/>
     </x:row>
-    <x:row r="23" ht="46" customHeight="1">
+    <x:row r="23" ht="72" customHeight="1">
       <x:c r="A23" s="48" t="str">
         <x:v>TG-0238</x:v>
       </x:c>
@@ -10075,7 +10075,7 @@
       </x:c>
       <x:c r="J23" s="48"/>
     </x:row>
-    <x:row r="24" ht="46" customHeight="1">
+    <x:row r="24" ht="72" customHeight="1">
       <x:c r="A24" s="48" t="str">
         <x:v>TG-0251</x:v>
       </x:c>
@@ -10089,7 +10089,7 @@
         <x:v>В треке Carefree, вышедшем в 2021 году, рэпер Songer занеймдроппил очень много футболистов. В одной из строчек он говорит, что у «Манчестер Сити» есть Рахим Стерлинг, но нет страйкера, поэтому клуб из Манчестера хочет ЕГО. За кем, по мнению Songer, охотился «Сити»?</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Эрлинг Холанд</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
         <x:v>https://t.me/simple_quiz/251</x:v>
@@ -10101,11 +10101,11 @@
         <x:v>0.956</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J24" s="48"/>
     </x:row>
-    <x:row r="25" ht="46" customHeight="1">
+    <x:row r="25" ht="72" customHeight="1">
       <x:c r="A25" s="48" t="str">
         <x:v>TG-0261</x:v>
       </x:c>
@@ -10119,7 +10119,7 @@
         <x:v>По состоянию на 2025 год Израиль, Кипр и Армения - единственные члены УЕФА, у которых нет ЭТОГО. О чем речь?</x:v>
       </x:c>
       <x:c r="E25" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Нахождение на территории Европы</x:v>
       </x:c>
       <x:c r="F25" s="50" t="str">
         <x:v>https://t.me/simple_quiz/261</x:v>
@@ -10131,11 +10131,11 @@
         <x:v>0.9191</x:v>
       </x:c>
       <x:c r="I25" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J25" s="48"/>
     </x:row>
-    <x:row r="26" ht="46" customHeight="1">
+    <x:row r="26" ht="72" customHeight="1">
       <x:c r="A26" s="48" t="str">
         <x:v>TG-0262</x:v>
       </x:c>
@@ -10149,7 +10149,7 @@
         <x:v>В сезоне-2025/26 в АПЛ их 7, в Чемпионшипе — 3, в английской Лиге 1 - 2, ав Лиге 2-1. О чем речь?</x:v>
       </x:c>
       <x:c r="E26" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Клубы из Лондона</x:v>
       </x:c>
       <x:c r="F26" s="50" t="str">
         <x:v>https://t.me/simple_quiz/262</x:v>
@@ -10161,11 +10161,11 @@
         <x:v>0.8598</x:v>
       </x:c>
       <x:c r="I26" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J26" s="48"/>
     </x:row>
-    <x:row r="27" ht="46" customHeight="1">
+    <x:row r="27" ht="72" customHeight="1">
       <x:c r="A27" s="48" t="str">
         <x:v>TG-0263</x:v>
       </x:c>
@@ -10179,7 +10179,7 @@
         <x:v>829 7” Sf о® Этот футболист провел всего год в «Дженоз», а потом укатил в Англию и следующие 8 лет играл исключительно в английских клубах. По окончании карьеры он тренировал клубы из восьми разных стран (и, в частности, работал в двух командах РПЛ). Аниме, в названии которого аж дважды содержится имя этого футболиста, прямо сейчас можно посмотреть в «Амедиатеке», а первые серии второго сезона летом показывали в московских кинотеатрах. Назовите этого футболиста. т WIN BOX od</x:v>
       </x:c>
       <x:c r="E27" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Дан Петреску</x:v>
       </x:c>
       <x:c r="F27" s="50" t="str">
         <x:v>https://t.me/simple_quiz/263</x:v>
@@ -10191,11 +10191,11 @@
         <x:v>0.9124</x:v>
       </x:c>
       <x:c r="I27" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J27" s="48"/>
     </x:row>
-    <x:row r="28" ht="46" customHeight="1">
+    <x:row r="28" ht="72" customHeight="1">
       <x:c r="A28" s="48" t="str">
         <x:v>TG-0264</x:v>
       </x:c>
@@ -10209,7 +10209,7 @@
         <x:v>9 2? Sf o° P Если записать названия клубов Ла Лиги с помощью элементов периодической таблицы, это получится с «Осасуной» (Os, As, Ц, Ма), «Бетисом» (Re, Al, Be, Ti, $) иеще одним клубом. В 2020 году этот клуб на один матч убрал из своего названия 4 буквы, оставив лишь Te, что с испанского переводятся как «вера», а в периодической таблице находятся на 26-м месте. Назовите этот клуб. — WIN вох ool</x:v>
       </x:c>
       <x:c r="E28" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Хетафе</x:v>
       </x:c>
       <x:c r="F28" s="50" t="str">
         <x:v>https://t.me/simple_quiz/264</x:v>
@@ -10221,11 +10221,11 @@
         <x:v>0.9046</x:v>
       </x:c>
       <x:c r="I28" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J28" s="48"/>
     </x:row>
-    <x:row r="29" ht="46" customHeight="1">
+    <x:row r="29" ht="72" customHeight="1">
       <x:c r="A29" s="48" t="str">
         <x:v>TG-0265</x:v>
       </x:c>
@@ -10239,7 +10239,7 @@
         <x:v>9 2? ve Va A о® АЛЬФА - вещь, которую видел или даже держал в руках каждый из вас. Один килограмм вяленых АЛЬФ можно найти на маркетплейсах за 3500 рублей, в то же время мешок АЛЬФ оценивают всего в 500 рублей. АЛЬФУ можно найти и на эмблеме одного из клубов Бундеслиги. Понять, какая именно АЛЬФА на эмблеме, просто: небольшой размер, округлая форма и направление вверх. Назовите АЛЬФУ. ее cnunmnn WIN BOX ool</x:v>
       </x:c>
       <x:c r="E29" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кедровая шишка</x:v>
       </x:c>
       <x:c r="F29" s="50" t="str">
         <x:v>https://t.me/simple_quiz/265</x:v>
@@ -10251,11 +10251,11 @@
         <x:v>0.8695</x:v>
       </x:c>
       <x:c r="I29" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J29" s="48"/>
     </x:row>
-    <x:row r="30" ht="46" customHeight="1">
+    <x:row r="30" ht="72" customHeight="1">
       <x:c r="A30" s="48" t="str">
         <x:v>TG-0285</x:v>
       </x:c>
@@ -10269,7 +10269,7 @@
         <x:v>Надпись на футболке этого футболиста в зависимости от эпохи и культурного контекста может означать как устройство для воспроизведения видео, так и последовательность чисел 5, 1, 500, 1, 100. Назовите этого футболиста.</x:v>
       </x:c>
       <x:c r="E30" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Неманья Видич</x:v>
       </x:c>
       <x:c r="F30" s="50" t="str">
         <x:v>https://t.me/simple_quiz/285</x:v>
@@ -10281,11 +10281,11 @@
         <x:v>0.9583</x:v>
       </x:c>
       <x:c r="I30" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J30" s="48"/>
     </x:row>
-    <x:row r="31" ht="46" customHeight="1">
+    <x:row r="31" ht="72" customHeight="1">
       <x:c r="A31" s="48" t="str">
         <x:v>TG-0286</x:v>
       </x:c>
@@ -10315,7 +10315,7 @@
       </x:c>
       <x:c r="J31" s="48"/>
     </x:row>
-    <x:row r="32" ht="46" customHeight="1">
+    <x:row r="32" ht="72" customHeight="1">
       <x:c r="A32" s="48" t="str">
         <x:v>TG-0291</x:v>
       </x:c>
@@ -10329,7 +10329,7 @@
         <x:v>ОМЕГА - локально культовый российский спортсмен не только благодаря результатам, но и благодаря ассоциации с трехзначным четным числом. Как только ты захотел спеть или сыграть музыкальное произведение с кем-то, ОМЕГА перестает быть ОМЕГОИ. Назовите ОМЕГУ.</x:v>
       </x:c>
       <x:c r="E32" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Соло 322</x:v>
       </x:c>
       <x:c r="F32" s="50" t="str">
         <x:v>https://t.me/simple_quiz/291</x:v>
@@ -10341,11 +10341,11 @@
         <x:v>0.9358</x:v>
       </x:c>
       <x:c r="I32" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J32" s="48"/>
     </x:row>
-    <x:row r="33" ht="46" customHeight="1">
+    <x:row r="33" ht="72" customHeight="1">
       <x:c r="A33" s="48" t="str">
         <x:v>TG-0294</x:v>
       </x:c>
@@ -10359,7 +10359,7 @@
         <x:v>Песня с названием «ИКС» вышла на альбоме 1999 года. 19 лет спустя та же группа выпустила песню «В ИКСЕ». Поклонники ИКСА поют ее на трибунах намного чаще. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E33" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Зенит</x:v>
       </x:c>
       <x:c r="F33" s="50" t="str">
         <x:v>https://t.me/simple_quiz/294</x:v>
@@ -10371,11 +10371,11 @@
         <x:v>0.962</x:v>
       </x:c>
       <x:c r="I33" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J33" s="48"/>
     </x:row>
-    <x:row r="34" ht="46" customHeight="1">
+    <x:row r="34" ht="72" customHeight="1">
       <x:c r="A34" s="48" t="str">
         <x:v>TG-0301</x:v>
       </x:c>
@@ -10389,7 +10389,7 @@
         <x:v>Из некоторых сокращений команд НХЛ получается слово на английском. Так, сокращение «Питтсбурга» — PIT — переводится как «яма», а сокращение «Сиэтла» - SEA - переводится как «море». Сокращения сразу двух клубов НХЛ в переводе означают транспортные средства. Назовите эти транспортные средства.</x:v>
       </x:c>
       <x:c r="E34" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Car и van</x:v>
       </x:c>
       <x:c r="F34" s="50" t="str">
         <x:v>https://t.me/simple_quiz/301</x:v>
@@ -10401,11 +10401,11 @@
         <x:v>0.9449</x:v>
       </x:c>
       <x:c r="I34" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J34" s="48"/>
     </x:row>
-    <x:row r="35" ht="46" customHeight="1">
+    <x:row r="35" ht="72" customHeight="1">
       <x:c r="A35" s="48" t="str">
         <x:v>TG-0302</x:v>
       </x:c>
@@ -10419,7 +10419,7 @@
         <x:v>В стандартной клавиатуре Windows 104 клавиши. Одна из них практически не используется в играх — в том числе и в той серии, название которой иллюстрирует. Например, в версии видеоигры 2021 года этой клавиши не было, а в версии 2025 года она по умолчанию обозначала «Extra Action 1». О какой клавише речь?</x:v>
       </x:c>
       <x:c r="E35" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="F35" s="50" t="str">
         <x:v>https://t.me/simple_quiz/302</x:v>
@@ -10431,11 +10431,11 @@
         <x:v>0.9565</x:v>
       </x:c>
       <x:c r="I35" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J35" s="48"/>
     </x:row>
-    <x:row r="36" ht="46" customHeight="1">
+    <x:row r="36" ht="72" customHeight="1">
       <x:c r="A36" s="48" t="str">
         <x:v>TG-0320</x:v>
       </x:c>
@@ -10449,7 +10449,7 @@
         <x:v>Псевдоним этого инди-исполнителя состоит из трех слов. Последние два описывают процесс, первое — ИКС: мужское имя в уменьшительной форме. Один из его самых популярных треков - «Волна». Также ИКС - разговорный синоним слова «команда». Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E36" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тима</x:v>
       </x:c>
       <x:c r="F36" s="50" t="str">
         <x:v>https://t.me/simple_quiz/320</x:v>
@@ -10461,11 +10461,11 @@
         <x:v>0.9469</x:v>
       </x:c>
       <x:c r="I36" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J36" s="48"/>
     </x:row>
-    <x:row r="37" ht="46" customHeight="1">
+    <x:row r="37" ht="72" customHeight="1">
       <x:c r="A37" s="48" t="str">
         <x:v>TG-0321</x:v>
       </x:c>
@@ -10479,7 +10479,7 @@
         <x:v>В 2022 году Василий Уткин говорил, что по утрам он обычно писал тексты, смотрел кино и даже делал зарядку. «Вы, наверное, удивитесь, но у меня дома есть ОНИ. И я ими пользуюсь по назначению», — рассказывал Василий. В отличие отлирического героя группы «Кровосток»: он пользовался ЕЙ не по назначению.</x:v>
       </x:c>
       <x:c r="E37" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Гантели</x:v>
       </x:c>
       <x:c r="F37" s="50" t="str">
         <x:v>https://t.me/simple_quiz/321</x:v>
@@ -10491,11 +10491,11 @@
         <x:v>0.9582</x:v>
       </x:c>
       <x:c r="I37" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J37" s="48"/>
     </x:row>
-    <x:row r="38" ht="46" customHeight="1">
+    <x:row r="38" ht="72" customHeight="1">
       <x:c r="A38" s="48" t="str">
         <x:v>TG-0325</x:v>
       </x:c>
@@ -10525,7 +10525,7 @@
       </x:c>
       <x:c r="J38" s="48"/>
     </x:row>
-    <x:row r="39" ht="46" customHeight="1">
+    <x:row r="39" ht="72" customHeight="1">
       <x:c r="A39" s="48" t="str">
         <x:v>TG-0326</x:v>
       </x:c>
@@ -10539,7 +10539,7 @@
         <x:v>В матчах ЦСКА можно стать свидетелем математического оксюморона. Его можно описать словосочетанием «ИКС ИГРЕКА». ИКС - часть фанатского сленга, а ИГРЕК - прозвище одного из футболистов ЦСКА. Назовите словосочетание, которое мы загадали.</x:v>
       </x:c>
       <x:c r="E39" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Угол круга</x:v>
       </x:c>
       <x:c r="F39" s="50" t="str">
         <x:v>https://t.me/simple_quiz/326</x:v>
@@ -10551,11 +10551,11 @@
         <x:v>0.9452</x:v>
       </x:c>
       <x:c r="I39" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J39" s="48"/>
     </x:row>
-    <x:row r="40" ht="46" customHeight="1">
+    <x:row r="40" ht="72" customHeight="1">
       <x:c r="A40" s="48" t="str">
         <x:v>TG-0327</x:v>
       </x:c>
@@ -10569,7 +10569,7 @@
         <x:v>Все мы подписываемся на блогеров или медиа в надежде получить кое-что качественное. ЭТОТ ИГРОК отличается от кое-чего наличием одной гласной буквы. Был ли ОН качественным - = вопрос дискуссионный, но 69 матчей за © 7 «Баварию» и 94 - за «Бордо» он провел О каком игроке идет речь? = i</x:v>
       </x:c>
       <x:c r="E40" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Контенто</x:v>
       </x:c>
       <x:c r="F40" s="50" t="str">
         <x:v>https://t.me/simple_quiz/327</x:v>
@@ -10581,11 +10581,11 @@
         <x:v>0.8689</x:v>
       </x:c>
       <x:c r="I40" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J40" s="48"/>
     </x:row>
-    <x:row r="41" ht="46" customHeight="1">
+    <x:row r="41" ht="72" customHeight="1">
       <x:c r="A41" s="48" t="str">
         <x:v>TG-0330</x:v>
       </x:c>
@@ -10599,7 +10599,7 @@
         <x:v>ИКС - российский бренд, который существует с 1995 года. Он специализируется на кетчупах, томатных пастах и уксусах. Сходить на ИКС у вас получится в НФЛ и MLB и не получится - в НХЛ, НБА и MLS. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E41" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Балтимор</x:v>
       </x:c>
       <x:c r="F41" s="50" t="str">
         <x:v>https://t.me/simple_quiz/330</x:v>
@@ -10611,11 +10611,11 @@
         <x:v>0.9414</x:v>
       </x:c>
       <x:c r="I41" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J41" s="48"/>
     </x:row>
-    <x:row r="42" ht="46" customHeight="1">
+    <x:row r="42" ht="72" customHeight="1">
       <x:c r="A42" s="48" t="str">
         <x:v>TG-0345</x:v>
       </x:c>
@@ -10645,7 +10645,7 @@
       </x:c>
       <x:c r="J42" s="48"/>
     </x:row>
-    <x:row r="43" ht="46" customHeight="1">
+    <x:row r="43" ht="72" customHeight="1">
       <x:c r="A43" s="48" t="str">
         <x:v>TG-0349</x:v>
       </x:c>
@@ -10675,7 +10675,7 @@
       </x:c>
       <x:c r="J43" s="48"/>
     </x:row>
-    <x:row r="44" ht="46" customHeight="1">
+    <x:row r="44" ht="72" customHeight="1">
       <x:c r="A44" s="48" t="str">
         <x:v>TG-0355</x:v>
       </x:c>
@@ -10689,7 +10689,7 @@
         <x:v>Когда хоккеиста Максима Афиногенова спросили про АЛЬФЫ, которые летят на лед во время матчей его команды, он ответил, что подобное встречается и в НХЛ, и привел пример с традицией в «Детройте» кидать на лед осьминога. Правда, если осьминог для «Ред Уингс» — победный символ, то АЛЬФА - оскорбление конкретной команды. Про что спросили после матча Макса Афиногенова?</x:v>
       </x:c>
       <x:c r="E44" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сосиски</x:v>
       </x:c>
       <x:c r="F44" s="50" t="str">
         <x:v>https://t.me/simple_quiz/355</x:v>
@@ -10701,11 +10701,11 @@
         <x:v>0.9544</x:v>
       </x:c>
       <x:c r="I44" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J44" s="48"/>
     </x:row>
-    <x:row r="45" ht="46" customHeight="1">
+    <x:row r="45" ht="72" customHeight="1">
       <x:c r="A45" s="48" t="str">
         <x:v>TG-0356</x:v>
       </x:c>
@@ -10719,7 +10719,7 @@
         <x:v>Несколько лет назад в интернете стало вирусным изображение одного ИКСа и Криштиану Роналду. Глядя на него, трудно поверить, что «ОМЕГА» ИКСА случилось позже - примерно через 308 дней после Роналду и через 474. года после «ОМЕГИ ИКСА» Микеланджело. Назовите, что такое ОМЕГА ИКСА.</x:v>
       </x:c>
       <x:c r="E45" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>«Сотворение Адама»</x:v>
       </x:c>
       <x:c r="F45" s="50" t="str">
         <x:v>https://t.me/simple_quiz/356</x:v>
@@ -10731,11 +10731,11 @@
         <x:v>0.9554</x:v>
       </x:c>
       <x:c r="I45" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J45" s="48"/>
     </x:row>
-    <x:row r="46" ht="46" customHeight="1">
+    <x:row r="46" ht="72" customHeight="1">
       <x:c r="A46" s="48" t="str">
         <x:v>TG-0367</x:v>
       </x:c>
@@ -10749,7 +10749,7 @@
         <x:v>Основное время семи матчей ЧМ-2018 закончилось со счетом, который можно записать, используя лишь имя одного из древних богов. Один из этих семи матчей, уверен, смотрел практически каждый из вас. Напишите счет этих матчей, используя лишь имя бога, но столько раз, сколько посчитаете нужным.</x:v>
       </x:c>
       <x:c r="E46" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>1:1</x:v>
       </x:c>
       <x:c r="F46" s="50" t="str">
         <x:v>https://t.me/simple_quiz/367</x:v>
@@ -10761,11 +10761,11 @@
         <x:v>0.9567</x:v>
       </x:c>
       <x:c r="I46" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J46" s="48"/>
     </x:row>
-    <x:row r="47" ht="46" customHeight="1">
+    <x:row r="47" ht="72" customHeight="1">
       <x:c r="A47" s="48" t="str">
         <x:v>TG-0371</x:v>
       </x:c>
@@ -10779,7 +10779,7 @@
         <x:v>С середины 2010-х несложно получить ретвит от одного из комментаторов Eurosport: достаточно сфотографировать автомобиль с этим трехзначным номером и отметить одного из комментаторов. Он почти всегда ретвитит фото с подобными номерами. Назовите трехзначное число, о котором мы рассказали в предыдущем абзаце.</x:v>
       </x:c>
       <x:c r="E47" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F47" s="50" t="str">
         <x:v>https://t.me/simple_quiz/371</x:v>
@@ -10791,11 +10791,11 @@
         <x:v>0.9549</x:v>
       </x:c>
       <x:c r="I47" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J47" s="48"/>
     </x:row>
-    <x:row r="48" ht="46" customHeight="1">
+    <x:row r="48" ht="72" customHeight="1">
       <x:c r="A48" s="48" t="str">
         <x:v>TG-0374</x:v>
       </x:c>
@@ -10809,7 +10809,7 @@
         <x:v>На «Википедии» можно найти свыше 30 различных ИКСОВ: это, например, и город в Калифорнии, и столица острова Тенерифе, и крупнейший город Боливии. Но мы помним другого ИКСА: того, что играл за «Баварию», «Манчестер Сити», «Блэкберн», «Малагу» и «Бетис». А еще - за мексиканский клуб, название которого ну очень ему подходит. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E48" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Санта-Крус</x:v>
       </x:c>
       <x:c r="F48" s="50" t="str">
         <x:v>https://t.me/simple_quiz/374</x:v>
@@ -10821,11 +10821,11 @@
         <x:v>0.9548</x:v>
       </x:c>
       <x:c r="I48" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J48" s="48"/>
     </x:row>
-    <x:row r="49" ht="46" customHeight="1">
+    <x:row r="49" ht="72" customHeight="1">
       <x:c r="A49" s="48" t="str">
         <x:v>TG-0387</x:v>
       </x:c>
@@ -10855,7 +10855,7 @@
       </x:c>
       <x:c r="J49" s="48"/>
     </x:row>
-    <x:row r="50" ht="46" customHeight="1">
+    <x:row r="50" ht="72" customHeight="1">
       <x:c r="A50" s="48" t="str">
         <x:v>TG-0388</x:v>
       </x:c>
@@ -10869,7 +10869,7 @@
         <x:v>ИКС - экс-футболист «Зенита», который, помимо России, поиграл в Германии, Греции, Турции, Венгрии и даже Австралии. ИКСЫ - картина Винсента ван Гога 1887 года. Кстати, в период карьеры в «Зените» у ИКСА не было на спине ни единицы, ни восьмерки, ни семерки. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E50" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мак</x:v>
       </x:c>
       <x:c r="F50" s="50" t="str">
         <x:v>https://t.me/simple_quiz/388</x:v>
@@ -10881,11 +10881,11 @@
         <x:v>0.9545</x:v>
       </x:c>
       <x:c r="I50" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J50" s="48"/>
     </x:row>
-    <x:row r="51" ht="46" customHeight="1">
+    <x:row r="51" ht="72" customHeight="1">
       <x:c r="A51" s="48" t="str">
         <x:v>TG-0392</x:v>
       </x:c>
@@ -10899,7 +10899,7 @@
         <x:v>Один ИКС изначально был не ИКСОМ, а Чейни. Другой ИКС раньше был не ИКСОМ, а Августой. Один ИКС периодически зарабатывал деньги боксом. Другой ИКС не раз принимал крупные боксерские поединки. Там дрались и Поветкин, и Кличко. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E51" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лондон</x:v>
       </x:c>
       <x:c r="F51" s="50" t="str">
         <x:v>https://t.me/simple_quiz/392</x:v>
@@ -10911,11 +10911,11 @@
         <x:v>0.9575</x:v>
       </x:c>
       <x:c r="I51" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J51" s="48"/>
     </x:row>
-    <x:row r="52" ht="46" customHeight="1">
+    <x:row r="52" ht="72" customHeight="1">
       <x:c r="A52" s="48" t="str">
         <x:v>TG-0399</x:v>
       </x:c>
@@ -10929,7 +10929,7 @@
         <x:v>Всю карьеру ОН выступал на резине бренда Light Year. В числе его спонсоров - Vitoline, Clutch+Aid, Mood Springs, Octane Gain, NitroAde, Easy Idle. Логотипы этих брендов можно увидеть Ha HEM. Назовите ЕГО двумя словами.</x:v>
       </x:c>
       <x:c r="E52" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Молния Маккуин</x:v>
       </x:c>
       <x:c r="F52" s="50" t="str">
         <x:v>https://t.me/simple_quiz/399</x:v>
@@ -10941,11 +10941,11 @@
         <x:v>0.9504</x:v>
       </x:c>
       <x:c r="I52" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J52" s="48"/>
     </x:row>
-    <x:row r="53" ht="46" customHeight="1">
+    <x:row r="53" ht="72" customHeight="1">
       <x:c r="A53" s="48" t="str">
         <x:v>TG-0415</x:v>
       </x:c>
@@ -10959,7 +10959,7 @@
         <x:v>Аккаунт nbaresdev выяснил, что игроки НБА начинают играть хуже после того, как обзаводятся ИМИ. В качестве доказательства они привели статистику Леброна Джеймса, Кевина Дюранта, Дреймонда Грина, Пола Джорджаи Джей Джея Редика. У всех них упали цифры по сезону после появления ИХ в их жизни. По одной из версий, первый ОН появился в 2004 году. В том же году это слово впервые использовал журналист Бен Хаммерсли. Кого мы зашифровали под НИМ?</x:v>
       </x:c>
       <x:c r="E53" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Подкаст</x:v>
       </x:c>
       <x:c r="F53" s="50" t="str">
         <x:v>https://t.me/simple_quiz/415</x:v>
@@ -10971,11 +10971,11 @@
         <x:v>0.9526</x:v>
       </x:c>
       <x:c r="I53" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J53" s="48"/>
     </x:row>
-    <x:row r="54" ht="46" customHeight="1">
+    <x:row r="54" ht="72" customHeight="1">
       <x:c r="A54" s="48" t="str">
         <x:v>TG-0417</x:v>
       </x:c>
@@ -10989,7 +10989,7 @@
         <x:v>Американская актриса Оливия Коберн известна многим из вас под другой фамилией. Одна из самых популярных сериальных ролей Оливии - ИКС. Догадаться, что мы спрятали под ИКСОМ, вам помогут Микаэль Баллак, Алессандро Неста и Майкон. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E54" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тринадцатая</x:v>
       </x:c>
       <x:c r="F54" s="50" t="str">
         <x:v>https://t.me/simple_quiz/417</x:v>
@@ -11001,11 +11001,11 @@
         <x:v>0.9522</x:v>
       </x:c>
       <x:c r="I54" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J54" s="48"/>
     </x:row>
-    <x:row r="55" ht="46" customHeight="1">
+    <x:row r="55" ht="72" customHeight="1">
       <x:c r="A55" s="48" t="str">
         <x:v>TG-0418</x:v>
       </x:c>
@@ -11019,7 +11019,7 @@
         <x:v>Бенджамин Франклин говорил, что не наблюдать за ИКСАМИ - значит, оставлять им открытым свой кошелек. Если к ИКСАМ добавить согласную букву, получится название футбольного клуба, который в августе 2005 года приезжал в Москву на матч с «Локомотивом». Назовите этот клуб.</x:v>
       </x:c>
       <x:c r="E55" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Работнички</x:v>
       </x:c>
       <x:c r="F55" s="50" t="str">
         <x:v>https://t.me/simple_quiz/418</x:v>
@@ -11031,11 +11031,11 @@
         <x:v>0.9565</x:v>
       </x:c>
       <x:c r="I55" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J55" s="48"/>
     </x:row>
-    <x:row r="56" ht="46" customHeight="1">
+    <x:row r="56" ht="72" customHeight="1">
       <x:c r="A56" s="48" t="str">
         <x:v>TG-0421</x:v>
       </x:c>
@@ -11049,7 +11049,7 @@
         <x:v>В 1978-1979 годах логотип «Нью-Йорк Никс» был в форме НЕГО. Вот некоторые ИХ представители: Fuji, Empire, Jonathan, Arkansas Black, Discovery. О чем речь?</x:v>
       </x:c>
       <x:c r="E56" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Яблоко</x:v>
       </x:c>
       <x:c r="F56" s="50" t="str">
         <x:v>https://t.me/simple_quiz/421</x:v>
@@ -11061,11 +11061,11 @@
         <x:v>0.958</x:v>
       </x:c>
       <x:c r="I56" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J56" s="48"/>
     </x:row>
-    <x:row r="57" ht="46" customHeight="1">
+    <x:row r="57" ht="72" customHeight="1">
       <x:c r="A57" s="48" t="str">
         <x:v>TG-0431</x:v>
       </x:c>
@@ -11079,7 +11079,7 @@
         <x:v>В ноябре 2022 года в соревновательный Counter-Strike добавили ИКС. Правда, уже через пару лет его убрали из про-сцены. Вы могли слышать про ИКСА на уроках истории. Если бы вы назвали ИКСА шакалом, это в какой-то степени было правдивым утверждением. В одной из древних культур он считался изобретателем бальзамирования. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E57" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Анубис</x:v>
       </x:c>
       <x:c r="F57" s="50" t="str">
         <x:v>https://t.me/simple_quiz/431</x:v>
@@ -11091,11 +11091,11 @@
         <x:v>0.9584</x:v>
       </x:c>
       <x:c r="I57" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J57" s="48"/>
     </x:row>
-    <x:row r="58" ht="46" customHeight="1">
+    <x:row r="58" ht="72" customHeight="1">
       <x:c r="A58" s="48" t="str">
         <x:v>TG-0434</x:v>
       </x:c>
@@ -11125,7 +11125,7 @@
       </x:c>
       <x:c r="J58" s="48"/>
     </x:row>
-    <x:row r="59" ht="46" customHeight="1">
+    <x:row r="59" ht="72" customHeight="1">
       <x:c r="A59" s="48" t="str">
         <x:v>TG-0437</x:v>
       </x:c>
@@ -11139,7 +11139,7 @@
         <x:v>К концу 2024 года в их списке есть и ЦСКА, и «Локомотив», и «Спартак», и «Динамо», иеще 267 других. «Торпедо» в их списке, кстати, нет. О чем речь?</x:v>
       </x:c>
       <x:c r="E59" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Станции Московского метрополитена</x:v>
       </x:c>
       <x:c r="F59" s="50" t="str">
         <x:v>https://t.me/simple_quiz/437</x:v>
@@ -11151,11 +11151,11 @@
         <x:v>0.9484</x:v>
       </x:c>
       <x:c r="I59" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J59" s="48"/>
     </x:row>
-    <x:row r="60" ht="46" customHeight="1">
+    <x:row r="60" ht="72" customHeight="1">
       <x:c r="A60" s="48" t="str">
         <x:v>TG-0438</x:v>
       </x:c>
@@ -11169,7 +11169,7 @@
         <x:v>В ребрендинге 2020 года одной национальной команды на эмблеме объединили четырех мифических хранителей — быка, орла, дракона и великана; новый знак заменил прежний щит с аббревиатурой федерации и флагом. Согласно пресс-релизу, эти фигуры - традиционные защитники страны и мотив, связанный с государственной символикой. Назовите сборную, которая впервые добралась до ЧМ и ЧЕ лишь в ХХ! веке.</x:v>
       </x:c>
       <x:c r="E60" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Исландия</x:v>
       </x:c>
       <x:c r="F60" s="50" t="str">
         <x:v>https://t.me/simple_quiz/438</x:v>
@@ -11181,11 +11181,11 @@
         <x:v>0.9522</x:v>
       </x:c>
       <x:c r="I60" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J60" s="48"/>
     </x:row>
-    <x:row r="61" ht="46" customHeight="1">
+    <x:row r="61" ht="72" customHeight="1">
       <x:c r="A61" s="48" t="str">
         <x:v>TG-0441</x:v>
       </x:c>
@@ -11199,7 +11199,7 @@
         <x:v>Шахматы 1922 года по модели Натальи Данько являются заметным образцом агитационного фарфора. В целях пропаганды скульптор придумала новые образы для каждой фигуры и заменила один из их традиционных цветов. Напишите пару цветов в версии шахмат Натальи Данько.</x:v>
       </x:c>
       <x:c r="E61" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Красные и белые</x:v>
       </x:c>
       <x:c r="F61" s="50" t="str">
         <x:v>https://t.me/simple_quiz/441</x:v>
@@ -11211,11 +11211,11 @@
         <x:v>0.9599</x:v>
       </x:c>
       <x:c r="I61" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J61" s="48"/>
     </x:row>
-    <x:row r="62" ht="46" customHeight="1">
+    <x:row r="62" ht="72" customHeight="1">
       <x:c r="A62" s="48" t="str">
         <x:v>TG-0445</x:v>
       </x:c>
@@ -11245,7 +11245,7 @@
       </x:c>
       <x:c r="J62" s="48"/>
     </x:row>
-    <x:row r="63" ht="46" customHeight="1">
+    <x:row r="63" ht="72" customHeight="1">
       <x:c r="A63" s="48" t="str">
         <x:v>TG-0450</x:v>
       </x:c>
@@ -11259,7 +11259,7 @@
         <x:v>Около 10 лет назад у очень многих сильных игроков в фифу была определенная особенность в никнейме, поэтому их называли ИКСАМИ. Позднее термин трансформировался, и ИКСАМИ стали называть всех сильных игроков вне зависимости от того, какой у них никнейм. ИКСОМ можно назвать, например, Мохамеда Салаха, Рияда Мареза или Ашрафа Хакими. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E63" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Араб</x:v>
       </x:c>
       <x:c r="F63" s="50" t="str">
         <x:v>https://t.me/simple_quiz/450</x:v>
@@ -11271,11 +11271,11 @@
         <x:v>0.9473</x:v>
       </x:c>
       <x:c r="I63" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J63" s="48"/>
     </x:row>
-    <x:row r="64" ht="46" customHeight="1">
+    <x:row r="64" ht="72" customHeight="1">
       <x:c r="A64" s="48" t="str">
         <x:v>TG-0451</x:v>
       </x:c>
@@ -11305,7 +11305,7 @@
       </x:c>
       <x:c r="J64" s="48"/>
     </x:row>
-    <x:row r="65" ht="46" customHeight="1">
+    <x:row r="65" ht="72" customHeight="1">
       <x:c r="A65" s="48" t="str">
         <x:v>TG-0452</x:v>
       </x:c>
@@ -11319,7 +11319,7 @@
         <x:v>В саундтреке FIFA 07 была песня этой группы. У этого трека 99 миллионов прослушиваний в Spotify, а у самой популярной песни группы - больше 2 миллиардов. Название этой группы совпадает с фамилиями двух легендарных игроков АПЛ. Один сыграл больше 200 матчей за «Тоттенхэм» и заезжал на сезон в «Ливерпуль». Другой провел больше 300 матчей за «МЮ». Как называется группа?</x:v>
       </x:c>
       <x:c r="E65" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Keane</x:v>
       </x:c>
       <x:c r="F65" s="50" t="str">
         <x:v>https://t.me/simple_quiz/452</x:v>
@@ -11331,11 +11331,11 @@
         <x:v>0.9569</x:v>
       </x:c>
       <x:c r="I65" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J65" s="48"/>
     </x:row>
-    <x:row r="66" ht="46" customHeight="1">
+    <x:row r="66" ht="72" customHeight="1">
       <x:c r="A66" s="48" t="str">
         <x:v>TG-0454</x:v>
       </x:c>
@@ -11349,7 +11349,7 @@
         <x:v>До 2006 года там не фигурировал никто, а после 2022-го там можно было увидеть следующих исполнителей: Drake, The Rolling Stones, Coldplay, Karol С, Rosalia, Travis Scott. В этом списке могли быть Тэйлор Свифт и Эд Ширан, но пока не срослось. Что объединяет вышеуказанных артистов?</x:v>
       </x:c>
       <x:c r="E66" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Игровые футболки «Барселоны»</x:v>
       </x:c>
       <x:c r="F66" s="50" t="str">
         <x:v>https://t.me/simple_quiz/454</x:v>
@@ -11361,11 +11361,11 @@
         <x:v>0.9576</x:v>
       </x:c>
       <x:c r="I66" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J66" s="48"/>
     </x:row>
-    <x:row r="67" ht="46" customHeight="1">
+    <x:row r="67" ht="72" customHeight="1">
       <x:c r="A67" s="48" t="str">
         <x:v>TG-0467</x:v>
       </x:c>
@@ -11379,7 +11379,7 @@
         <x:v>Дженнифер Лоуренс, Орландо Блум, Джереми Реннер, Рассел Кроу, Стивен Амелл - всех этих актеров объединяет некий олимпийский вид спорта. Назовите этот вид спорта.</x:v>
       </x:c>
       <x:c r="E67" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Стрельба из лука</x:v>
       </x:c>
       <x:c r="F67" s="50" t="str">
         <x:v>https://t.me/simple_quiz/467</x:v>
@@ -11391,11 +11391,11 @@
         <x:v>0.9541</x:v>
       </x:c>
       <x:c r="I67" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J67" s="48"/>
     </x:row>
-    <x:row r="68" ht="46" customHeight="1">
+    <x:row r="68" ht="72" customHeight="1">
       <x:c r="A68" s="48" t="str">
         <x:v>TG-0468</x:v>
       </x:c>
@@ -11409,7 +11409,7 @@
         <x:v>Перед вами зашифрован персонаж культового произведения английского писателя. Мы уверены, что сам персонаж с легкостью прочел бы указанный SYXFRR EK Sete Однофамилец этого персонажа провел 10 сезонов в НБА. Он поиграл в «Филадельфии», «Финиксе», «Сакраменто», «Далласе» и «Вашингтоне». Он до сих пор в лиге. Назовите фамилию персонажа. Или баскетболиста.</x:v>
       </x:c>
       <x:c r="E68" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Шерлок Холмс</x:v>
       </x:c>
       <x:c r="F68" s="50" t="str">
         <x:v>https://t.me/simple_quiz/468</x:v>
@@ -11421,11 +11421,11 @@
         <x:v>0.9021</x:v>
       </x:c>
       <x:c r="I68" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J68" s="48"/>
     </x:row>
-    <x:row r="69" ht="46" customHeight="1">
+    <x:row r="69" ht="72" customHeight="1">
       <x:c r="A69" s="48" t="str">
         <x:v>TG-0469</x:v>
       </x:c>
@@ -11439,7 +11439,7 @@
         <x:v>В США расфорсился скриншот с матча МЛБ между «Чикаго Кабс» и «Питтсбургом». На этом скриншоте видны упрощенные лого команд- участниц и счет матча, в котором одна из команд пока не набрала очков. Символы на этом скриншоте повторяют имя персонажа, фигурировавшего во всех эпизодах известнейшей франшизы. Напишите имя этого персонажа.</x:v>
       </x:c>
       <x:c r="E69" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>C-3PO</x:v>
       </x:c>
       <x:c r="F69" s="50" t="str">
         <x:v>https://t.me/simple_quiz/469</x:v>
@@ -11451,11 +11451,11 @@
         <x:v>0.9542</x:v>
       </x:c>
       <x:c r="I69" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J69" s="48"/>
     </x:row>
-    <x:row r="70" ht="46" customHeight="1">
+    <x:row r="70" ht="72" customHeight="1">
       <x:c r="A70" s="48" t="str">
         <x:v>TG-0473</x:v>
       </x:c>
@@ -11469,7 +11469,7 @@
         <x:v>ИКС ИГРЕК - двукратный чемпион НБА, бронзовый призер Олимпийских игр и чемпион мира. ИКС ЗЕТ - звезда НФЛ, которая с 2019 года играет в одной команде. ИПСИЛОН ИКС - обладатель 22 наград «Грэмми». С НФЛ он так или иначе тоже связан. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E70" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Ламар</x:v>
       </x:c>
       <x:c r="F70" s="50" t="str">
         <x:v>https://t.me/simple_quiz/473</x:v>
@@ -11481,11 +11481,11 @@
         <x:v>0.9493</x:v>
       </x:c>
       <x:c r="I70" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J70" s="48"/>
     </x:row>
-    <x:row r="71" ht="46" customHeight="1">
+    <x:row r="71" ht="72" customHeight="1">
       <x:c r="A71" s="48" t="str">
         <x:v>TG-0474</x:v>
       </x:c>
@@ -11499,7 +11499,7 @@
         <x:v>После поражения сборной Англии по крикету от Австралии в 1882 году The Sporting Times напечатали некролог: «Английский крикет умер 29 августа 1882 года». С тех пор победителям серии матчей между Англией и Австралией в тестовом крикете вручается ОНА. Возможно, если бы EE подарили вам, это вызвало быу вас как минимум непонимание, ау некоторых - даже обиду. Назовите EE двумя словами.</x:v>
       </x:c>
       <x:c r="E71" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Урна</x:v>
       </x:c>
       <x:c r="F71" s="50" t="str">
         <x:v>https://t.me/simple_quiz/474</x:v>
@@ -11511,11 +11511,11 @@
         <x:v>0.9563</x:v>
       </x:c>
       <x:c r="I71" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J71" s="48"/>
     </x:row>
-    <x:row r="72" ht="46" customHeight="1">
+    <x:row r="72" ht="72" customHeight="1">
       <x:c r="A72" s="48" t="str">
         <x:v>TG-0505</x:v>
       </x:c>
@@ -11529,7 +11529,7 @@
         <x:v>Один из текстов на сайте Eurosport.ru, посвященный триумфу одной биатлонистки, был озаглавлен «ОНА маслом». ОНА - фамилия спортсменки, забравшейся на подиум. Назовите ЕЕ.</x:v>
       </x:c>
       <x:c r="E72" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Надежда Скардино</x:v>
       </x:c>
       <x:c r="F72" s="50" t="str">
         <x:v>https://t.me/simple_quiz/505</x:v>
@@ -11541,11 +11541,11 @@
         <x:v>0.941</x:v>
       </x:c>
       <x:c r="I72" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J72" s="48"/>
     </x:row>
-    <x:row r="73" ht="46" customHeight="1">
+    <x:row r="73" ht="72" customHeight="1">
       <x:c r="A73" s="48" t="str">
         <x:v>TG-0507</x:v>
       </x:c>
@@ -11559,7 +11559,7 @@
         <x:v>Перед вами список спортсменов: легкоатлет Ноа Лайлз, гольфист Брайсон Дешамбо, теннисистка Серена Уильямс, бейсболист Аарон Джадж, футболисты Неймар и Криштиану Роналду, баскетболисты Стефен Карри и Дэмиан Лиллард. В 2024 и 2025 гг. их медийно объединил один человек 1998 года рождения, чье настоящее имя — Джеймс Стивен Дональдсон. Назовите псевдоним этого человека.</x:v>
       </x:c>
       <x:c r="E73" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>MrBeast</x:v>
       </x:c>
       <x:c r="F73" s="50" t="str">
         <x:v>https://t.me/simple_quiz/507</x:v>
@@ -11571,11 +11571,11 @@
         <x:v>0.9451</x:v>
       </x:c>
       <x:c r="I73" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J73" s="48"/>
     </x:row>
-    <x:row r="74" ht="46" customHeight="1">
+    <x:row r="74" ht="72" customHeight="1">
       <x:c r="A74" s="48" t="str">
         <x:v>TG-0508</x:v>
       </x:c>
@@ -11589,7 +11589,7 @@
         <x:v>Имена Диего Марадоны, Майка Тайсона, Роналдиньо, Флойда Мэйуэзера, Аллена Айверсона фигурировали в различных ИХ. В архитектуре ОН, помимо самых известных, бывает коринфским или тосканским. Назовите ЕГО.</x:v>
       </x:c>
       <x:c r="E74" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Ордер</x:v>
       </x:c>
       <x:c r="F74" s="50" t="str">
         <x:v>https://t.me/simple_quiz/508</x:v>
@@ -11601,11 +11601,11 @@
         <x:v>0.9508</x:v>
       </x:c>
       <x:c r="I74" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J74" s="48"/>
     </x:row>
-    <x:row r="75" ht="46" customHeight="1">
+    <x:row r="75" ht="72" customHeight="1">
       <x:c r="A75" s="48" t="str">
         <x:v>TG-0509</x:v>
       </x:c>
@@ -11619,7 +11619,7 @@
         <x:v>Эта аббревиатура в какой-то степени ассоциируется с темнокожими людьми, правда, не в спортивных медиа, а в диджитал-файлах совершенно другого типа. A еще эта аббревиатура - название медиа, у которого есть не только спортивный раздел, но и целое пан- Африканское направление и редакция. Воспроизведите эту аббревиатуру, состоящую из трех латинских букв.</x:v>
       </x:c>
       <x:c r="E75" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>BBC</x:v>
       </x:c>
       <x:c r="F75" s="50" t="str">
         <x:v>https://t.me/simple_quiz/509</x:v>
@@ -11631,11 +11631,11 @@
         <x:v>0.9486</x:v>
       </x:c>
       <x:c r="I75" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J75" s="48"/>
     </x:row>
-    <x:row r="76" ht="46" customHeight="1">
+    <x:row r="76" ht="72" customHeight="1">
       <x:c r="A76" s="48" t="str">
         <x:v>TG-0511</x:v>
       </x:c>
@@ -11649,7 +11649,7 @@
         <x:v>В романтическом плане Матвея Сафонова можно назвать ИМ - например, для его жены Марины. OH на французском языке — фамилия одного из партнеров Сафонова. Также ОН во Франции- низшая категория ордена Почетного легиона. Назовите ЕГО французским словом.</x:v>
       </x:c>
       <x:c r="E76" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Chevalier (шевалье)</x:v>
       </x:c>
       <x:c r="F76" s="50" t="str">
         <x:v>https://t.me/simple_quiz/511</x:v>
@@ -11661,11 +11661,11 @@
         <x:v>0.949</x:v>
       </x:c>
       <x:c r="I76" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J76" s="48"/>
     </x:row>
-    <x:row r="77" ht="46" customHeight="1">
+    <x:row r="77" ht="72" customHeight="1">
       <x:c r="A77" s="48" t="str">
         <x:v>TG-0512</x:v>
       </x:c>
@@ -11679,7 +11679,7 @@
         <x:v>В Северной Америке ТАК называют скамейки на матчах по бейсболу и американскому футболу, а также зрителей на этих играх. Одна из версий происхождения термина - что деревянные скамейки выгорали или выцветали на солнце. Также ЭТО СЛОВО присутствует в названии американского спортивного медиа, основанного в 2005 году. По сути, первые тексты создателей сайта стали взглядом с этих самых скамеек. Назовите слово или спортивное медиа.</x:v>
       </x:c>
       <x:c r="E77" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Bleachers</x:v>
       </x:c>
       <x:c r="F77" s="50" t="str">
         <x:v>https://t.me/simple_quiz/512</x:v>
@@ -11691,11 +11691,11 @@
         <x:v>0.9584</x:v>
       </x:c>
       <x:c r="I77" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J77" s="48"/>
     </x:row>
-    <x:row r="78" ht="46" customHeight="1">
+    <x:row r="78" ht="72" customHeight="1">
       <x:c r="A78" s="48" t="str">
         <x:v>TG-0514</x:v>
       </x:c>
@@ -11709,7 +11709,7 @@
         <x:v>Если бы Артем Дзюба провел всю карьеру в «Спартаке», то из-за одного факта биографии форварда на «Лукойл Арене» его могли бы называть ИКСом. ИКС - прозвище заметного политического деятеля, который жил в России на стыке 16-го и Т7-го веков. Назовите ИКС двумя словами.</x:v>
       </x:c>
       <x:c r="E78" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Тушинский вор</x:v>
       </x:c>
       <x:c r="F78" s="50" t="str">
         <x:v>https://t.me/simple_quiz/514</x:v>
@@ -11721,11 +11721,11 @@
         <x:v>0.9529</x:v>
       </x:c>
       <x:c r="I78" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J78" s="48"/>
     </x:row>
-    <x:row r="79" ht="46" customHeight="1">
+    <x:row r="79" ht="72" customHeight="1">
       <x:c r="A79" s="48" t="str">
         <x:v>TG-0516</x:v>
       </x:c>
@@ -11739,7 +11739,7 @@
         <x:v>В топ-100 прямых эфиров на американском телевидении в 2023 году вошли сразу 97 спортивных трансляций. 94 из них - это матчи NFL. A 3 оставшихся?</x:v>
       </x:c>
       <x:c r="E79" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>NCAA</x:v>
       </x:c>
       <x:c r="F79" s="50" t="str">
         <x:v>https://t.me/simple_quiz/516</x:v>
@@ -11751,11 +11751,11 @@
         <x:v>0.9452</x:v>
       </x:c>
       <x:c r="I79" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J79" s="48"/>
     </x:row>
-    <x:row r="80" ht="46" customHeight="1">
+    <x:row r="80" ht="72" customHeight="1">
       <x:c r="A80" s="48" t="str">
         <x:v>TG-0517</x:v>
       </x:c>
@@ -11769,7 +11769,7 @@
         <x:v>Карьера Сергея Юрьевича началась в клубе из Узбекистана в 1991 году, а завершилась в 2018 году в клубе из Белгорода. Сергей Юрьевич - олимпийский чемпион. Карьера Павла Сергеевича началась в 2017 году в клубе из Белгорода. Назовите фамилию Сергея Юрьевича и Павла Сергеевича.</x:v>
       </x:c>
       <x:c r="E80" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сергей Тетюхин</x:v>
       </x:c>
       <x:c r="F80" s="50" t="str">
         <x:v>https://t.me/simple_quiz/517</x:v>
@@ -11781,11 +11781,11 @@
         <x:v>0.9564</x:v>
       </x:c>
       <x:c r="I80" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J80" s="48"/>
     </x:row>
-    <x:row r="81" ht="46" customHeight="1">
+    <x:row r="81" ht="72" customHeight="1">
       <x:c r="A81" s="48" t="str">
         <x:v>TG-0518</x:v>
       </x:c>
@@ -11799,7 +11799,7 @@
         <x:v>В 1999 году «Манчестер Сити» подписал контракт с издательством Eidos Interactive. С анонса того соглашения осталось несколько фотографий с НЕЙ. В 2020 году сайт Coop-Land признал EE грудь лучшей в истории индустрии. Кого мы загадали под НЕЙ?</x:v>
       </x:c>
       <x:c r="E81" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лара Крофт</x:v>
       </x:c>
       <x:c r="F81" s="50" t="str">
         <x:v>https://t.me/simple_quiz/518</x:v>
@@ -11811,11 +11811,11 @@
         <x:v>0.9483</x:v>
       </x:c>
       <x:c r="I81" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J81" s="48"/>
     </x:row>
-    <x:row r="82" ht="46" customHeight="1">
+    <x:row r="82" ht="72" customHeight="1">
       <x:c r="A82" s="48" t="str">
         <x:v>TG-0519</x:v>
       </x:c>
@@ -11829,7 +11829,7 @@
         <x:v>В одном из спешалов комик Эндрю Шульц рассуждал о разнице между Чикаго и Нью-Иорком. Он обратил внимание, что, в отличие от нью-йоркцев, жители Чикаго гордятся трагедиями в городе настолько, что даже назвали команду по футболу - «Чикаго Файр» -— якобы в честь великого чикагского пожара 1871 года. Когда Шульц начал рассуждать о названиях команд в Нью- Иорке, зал взорвался от смеха. Название какой команды вызвало у зрителей истерику?</x:v>
       </x:c>
       <x:c r="E82" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Jets</x:v>
       </x:c>
       <x:c r="F82" s="50" t="str">
         <x:v>https://t.me/simple_quiz/519</x:v>
@@ -11841,11 +11841,11 @@
         <x:v>0.9458</x:v>
       </x:c>
       <x:c r="I82" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J82" s="48"/>
     </x:row>
-    <x:row r="83" ht="46" customHeight="1">
+    <x:row r="83" ht="72" customHeight="1">
       <x:c r="A83" s="48" t="str">
         <x:v>TG-0520</x:v>
       </x:c>
@@ -11859,7 +11859,7 @@
         <x:v>Блогер Софья Шамсутдинова ведет блог на «Спортсе”» и снимает рилзы Ha тему того, как учится играть в футбол: в роликах она чеканит мяч и делает разнообразные трюки. Название ее блога - каламбур, связанный сее именем и хорватским ресурсом, помогающим следить за ходом матча. Воспроизведите ее никнейм на «Спортсе”» и в других соцсетях.</x:v>
       </x:c>
       <x:c r="E83" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Sofascore</x:v>
       </x:c>
       <x:c r="F83" s="50" t="str">
         <x:v>https://t.me/simple_quiz/520</x:v>
@@ -11871,11 +11871,11 @@
         <x:v>0.9383</x:v>
       </x:c>
       <x:c r="I83" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J83" s="48"/>
     </x:row>
-    <x:row r="84" ht="46" customHeight="1">
+    <x:row r="84" ht="72" customHeight="1">
       <x:c r="A84" s="48" t="str">
         <x:v>TG-0521</x:v>
       </x:c>
@@ -11905,7 +11905,7 @@
       </x:c>
       <x:c r="J84" s="48"/>
     </x:row>
-    <x:row r="85" ht="46" customHeight="1">
+    <x:row r="85" ht="72" customHeight="1">
       <x:c r="A85" s="48" t="str">
         <x:v>TG-0524</x:v>
       </x:c>
@@ -11919,7 +11919,7 @@
         <x:v>Фотограф Денис Тырин опубликовал фотографию с турнира по фигурному катанию. Благодаря талантливому кадрированию фото от названия турнира на рекламном щите за спиной Аделии Петросян осталось лишь шесть букв, что добавило фотографии дополнительный смысл. Эти шесть букв вы можете найти даже в первом абзаце вопроса. Напишите их.</x:v>
       </x:c>
       <x:c r="E85" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Пофигу</x:v>
       </x:c>
       <x:c r="F85" s="50" t="str">
         <x:v>https://t.me/simple_quiz/524</x:v>
@@ -11931,11 +11931,11 @@
         <x:v>0.9588</x:v>
       </x:c>
       <x:c r="I85" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J85" s="48"/>
     </x:row>
-    <x:row r="86" ht="46" customHeight="1">
+    <x:row r="86" ht="72" customHeight="1">
       <x:c r="A86" s="48" t="str">
         <x:v>TG-0527</x:v>
       </x:c>
@@ -11949,7 +11949,7 @@
         <x:v>ИКС - фамилия довольно известного монстра. Если к ИКСУ добавить гласную букву и еще один орфографический знак, получится совершенно другой монстр: семикратный чемпион мира, выступающий на про-уровне вот уже 33 года. Назовите вид спорта, в котором выступает второй монстр.</x:v>
       </x:c>
       <x:c r="E86" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Снукер</x:v>
       </x:c>
       <x:c r="F86" s="50" t="str">
         <x:v>https://t.me/simple_quiz/527</x:v>
@@ -11961,11 +11961,11 @@
         <x:v>0.9528</x:v>
       </x:c>
       <x:c r="I86" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J86" s="48"/>
     </x:row>
-    <x:row r="87" ht="46" customHeight="1">
+    <x:row r="87" ht="72" customHeight="1">
       <x:c r="A87" s="48" t="str">
         <x:v>TG-0535</x:v>
       </x:c>
@@ -11979,7 +11979,7 @@
         <x:v>Среди экс-комментаторов «НТВ-Плюс», оказавшихся на «Матч ТВ», пригласили и ЗАМЕНА. ЗАМЕНА - один из футболистов «Комо». Игрок проводит лишь первый сезон в Серии А после трансфера из загребского «Динамо». Что мы зашифровали под ЗАМЕНА?</x:v>
       </x:c>
       <x:c r="E87" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Батурина</x:v>
       </x:c>
       <x:c r="F87" s="50" t="str">
         <x:v>https://t.me/simple_quiz/535</x:v>
@@ -11991,11 +11991,11 @@
         <x:v>0.9521</x:v>
       </x:c>
       <x:c r="I87" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J87" s="48"/>
     </x:row>
-    <x:row r="88" ht="46" customHeight="1">
+    <x:row r="88" ht="72" customHeight="1">
       <x:c r="A88" s="48" t="str">
         <x:v>TG-0542</x:v>
       </x:c>
@@ -12009,7 +12009,7 @@
         <x:v>В диджитал-версии журнала «Коммерсантъ» публикация, посвященная победе Андрея Рублева над Роджером Федерером, была озаглавлена следующим образом: «Андрей Рублев СДЕЛАЛ ЭТО». В 1904 году в Казанском Богородицком монастыре СДЕЛАЛИ ЭТО - это один из самых известных подобных случаев в России. Закончите заголовок «Коммерсанта» двумя словами.</x:v>
       </x:c>
       <x:c r="E88" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Вынес икону</x:v>
       </x:c>
       <x:c r="F88" s="50" t="str">
         <x:v>https://t.me/simple_quiz/542</x:v>
@@ -12021,11 +12021,11 @@
         <x:v>0.9577</x:v>
       </x:c>
       <x:c r="I88" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J88" s="48"/>
     </x:row>
-    <x:row r="89" ht="46" customHeight="1">
+    <x:row r="89" ht="72" customHeight="1">
       <x:c r="A89" s="48" t="str">
         <x:v>TG-0544</x:v>
       </x:c>
@@ -12039,7 +12039,7 @@
         <x:v>Довольно известный русский иконописец ИКС родился и вырос в Византии, поэтому вошел в историю как ИКС ИГРЕК. Сразу 23 чемпиона Европы по футболу в 21-м веке были ИГРЕКАМИ. Назовите ИГРЕК.</x:v>
       </x:c>
       <x:c r="E89" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Феофан Грек</x:v>
       </x:c>
       <x:c r="F89" s="50" t="str">
         <x:v>https://t.me/simple_quiz/544</x:v>
@@ -12051,11 +12051,11 @@
         <x:v>0.9529</x:v>
       </x:c>
       <x:c r="I89" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J89" s="48"/>
     </x:row>
-    <x:row r="90" ht="46" customHeight="1">
+    <x:row r="90" ht="72" customHeight="1">
       <x:c r="A90" s="48" t="str">
         <x:v>TG-0545</x:v>
       </x:c>
@@ -12069,7 +12069,7 @@
         <x:v>В средневековье во время осады города вражескими войсками в населенном пункте зачастую начинался ОН. Вы можете знать другого ЕГО: он периодически появляется в студии «Матч ТВ». Назовите ЕГО.</x:v>
       </x:c>
       <x:c r="E90" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мор</x:v>
       </x:c>
       <x:c r="F90" s="50" t="str">
         <x:v>https://t.me/simple_quiz/545</x:v>
@@ -12081,11 +12081,11 @@
         <x:v>0.9621</x:v>
       </x:c>
       <x:c r="I90" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J90" s="48"/>
     </x:row>
-    <x:row r="91" ht="46" customHeight="1">
+    <x:row r="91" ht="72" customHeight="1">
       <x:c r="A91" s="48" t="str">
         <x:v>TG-0551</x:v>
       </x:c>
@@ -12099,7 +12099,7 @@
         <x:v>ИИ-художник jslayart составил несколько ростеров по определенному принципу. В одну команду вошли Джейлен Брансон, Наруто, Гоку, Существо, Микеланджело, Аанг. В другую - Патрик Махоумс, Майкл Джордан, Флеш, Тайгер Вудс, Дэдпул. В третью - Ламар Джексон, TaHoc, Джокер, Канг Завоеватель, Фриза. По какому принципу составлены эти ростеры?</x:v>
       </x:c>
       <x:c r="E91" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>По цветам костюмов: оранжевый, красный, фиолетовый</x:v>
       </x:c>
       <x:c r="F91" s="50" t="str">
         <x:v>https://t.me/simple_quiz/551</x:v>
@@ -12111,11 +12111,11 @@
         <x:v>0.941</x:v>
       </x:c>
       <x:c r="I91" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J91" s="48"/>
     </x:row>
-    <x:row r="92" ht="46" customHeight="1">
+    <x:row r="92" ht="72" customHeight="1">
       <x:c r="A92" s="48" t="str">
         <x:v>TG-0552</x:v>
       </x:c>
@@ -12129,7 +12129,7 @@
         <x:v>В январе 2013 года Ha Sports.ru вышел пост Кирилла Благова, посвященный лишнему весу звезды РПЛ из Эквадора. Вторая часть заголовка выглядела так: «Как отпуск Кайседо превратился в событие». Первая состояла из имени и фамилии известного южноамериканского спортсмена. Воспроизведите каламбур из первой части заголовка.</x:v>
       </x:c>
       <x:c r="E92" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Фелипе Масса</x:v>
       </x:c>
       <x:c r="F92" s="50" t="str">
         <x:v>https://t.me/simple_quiz/552</x:v>
@@ -12141,11 +12141,11 @@
         <x:v>0.9534</x:v>
       </x:c>
       <x:c r="I92" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J92" s="48"/>
     </x:row>
-    <x:row r="93" ht="46" customHeight="1">
+    <x:row r="93" ht="72" customHeight="1">
       <x:c r="A93" s="48" t="str">
         <x:v>TG-0553</x:v>
       </x:c>
@@ -12159,7 +12159,7 @@
         <x:v>Серхио Перес, Сергей Карякин, Артур Шилов - всех их называли ИМ. Маурицио Сарри называл ИМ Лучано Спаллетти. Действующего ЕГО мы называть не будем. Назовите ЕГО двумя словами.</x:v>
       </x:c>
       <x:c r="E93" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Министр обороны</x:v>
       </x:c>
       <x:c r="F93" s="50" t="str">
         <x:v>https://t.me/simple_quiz/553</x:v>
@@ -12171,11 +12171,11 @@
         <x:v>0.956</x:v>
       </x:c>
       <x:c r="I93" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J93" s="48"/>
     </x:row>
-    <x:row r="94" ht="46" customHeight="1">
+    <x:row r="94" ht="72" customHeight="1">
       <x:c r="A94" s="48" t="str">
         <x:v>TG-0555</x:v>
       </x:c>
@@ -12189,7 +12189,7 @@
         <x:v>ОНО - один из самых популярных фильмов Брайана Де Пальмы. ОНО - прозвище культового футболиста, который отбегал 17 матчей за «Галатасарай», а потом 17 лет играл исключительно в клубах из топ-5 лиг Европы. Что такое ОНО? Ответьте тремя словами.</x:v>
       </x:c>
       <x:c r="E94" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лицо со шрамом</x:v>
       </x:c>
       <x:c r="F94" s="50" t="str">
         <x:v>https://t.me/simple_quiz/555</x:v>
@@ -12201,11 +12201,11 @@
         <x:v>0.9556</x:v>
       </x:c>
       <x:c r="I94" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J94" s="48"/>
     </x:row>
-    <x:row r="95" ht="46" customHeight="1">
+    <x:row r="95" ht="72" customHeight="1">
       <x:c r="A95" s="48" t="str">
         <x:v>TG-0561</x:v>
       </x:c>
@@ -12219,7 +12219,7 @@
         <x:v>_—— ss В 2021 году в Германии выпустили 110 почтовые марки, посвященные 25- о к Fa С летнему юбилею победы ЕГО a АА. ag м4 *у над действующим на тот момент им а ем 3 тг AS dy Hye чемпионом мира Гарри Каспаровым. и мм “a ast i Несмотря на то, что мы скрыли 2 ЖЕ! фрагмент марки, вы все равно можете a F рассмотреть ЕГО на изображении. САВЕ! KASPAROW 20216 Назовите ЕГО имя двумя английскими словами абсолютно точно.</x:v>
       </x:c>
       <x:c r="E95" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Deep Blue</x:v>
       </x:c>
       <x:c r="F95" s="50" t="str">
         <x:v>https://t.me/simple_quiz/561</x:v>
@@ -12231,11 +12231,11 @@
         <x:v>0.7426</x:v>
       </x:c>
       <x:c r="I95" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J95" s="48"/>
     </x:row>
-    <x:row r="96" ht="46" customHeight="1">
+    <x:row r="96" ht="72" customHeight="1">
       <x:c r="A96" s="48" t="str">
         <x:v>TG-0567</x:v>
       </x:c>
@@ -12249,7 +12249,7 @@
         <x:v>В США начали принимать ставки на то, кто СДЕЛАЕТ ЭТО до 2027 года. Иронично, что шансы на то, что Леброн Джеймс СДЕЛАЕТ ЭТО до 2027 года, оценивают выше, чем шансы на чемпионство «Лейкерс». Согласно котировкам букмекеров, шансы Леброна на то, что он СДЕЛАЕТ ЭТО до 2027 года, ниже, чем, например, владельца «Далласа» Марка Кьюбана, экс-игрока НФЛ Тома Брэйди, спортивного аналитика Стивена Эй Смита, а еще - Дуэйна «Скалы» Джонсона, Джорджа Клуни, Илона Маска и Ким Кардашьян. Что мы зашифровали под СДЕЛАЕТ ЭТО?</x:v>
       </x:c>
       <x:c r="E96" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Объявит о выдвижении в президенты</x:v>
       </x:c>
       <x:c r="F96" s="50" t="str">
         <x:v>https://t.me/simple_quiz/567</x:v>
@@ -12261,11 +12261,11 @@
         <x:v>0.9525</x:v>
       </x:c>
       <x:c r="I96" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J96" s="48"/>
     </x:row>
-    <x:row r="97" ht="46" customHeight="1">
+    <x:row r="97" ht="72" customHeight="1">
       <x:c r="A97" s="48" t="str">
         <x:v>TG-0568</x:v>
       </x:c>
@@ -12279,7 +12279,7 @@
         <x:v>В 1921 году британец Гарольд Сирлс Торнтон запатентовал некое устройство. Его структуру можно описать числовым рядом «123553 2 I». Сейчас многие из вас знают это устройство как ИКС Другой ИКС, который вы тоже можете знать, был основан на год раньше, в 1920 году в Нюрнберге. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E97" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кикер</x:v>
       </x:c>
       <x:c r="F97" s="50" t="str">
         <x:v>https://t.me/simple_quiz/568</x:v>
@@ -12291,11 +12291,11 @@
         <x:v>0.9548</x:v>
       </x:c>
       <x:c r="I97" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J97" s="48"/>
     </x:row>
-    <x:row r="98" ht="46" customHeight="1">
+    <x:row r="98" ht="72" customHeight="1">
       <x:c r="A98" s="48" t="str">
         <x:v>TG-0569</x:v>
       </x:c>
@@ -12309,7 +12309,7 @@
         <x:v>В 2008 году сайт Goal.com опубликовал пост, посвященный поражению «Ювентуса» в еврокубковом матче. Он звучал на английском так: «Old Lady unable to master ПРОПУСК at home». Разумеется, в заголовке зашифрована игра слов, причем довольно непристойная. Заполните ПРОПУСК четырьмя буквами.</x:v>
       </x:c>
       <x:c r="E98" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>БАТЭ</x:v>
       </x:c>
       <x:c r="F98" s="50" t="str">
         <x:v>https://t.me/simple_quiz/569</x:v>
@@ -12321,11 +12321,11 @@
         <x:v>0.9497</x:v>
       </x:c>
       <x:c r="I98" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J98" s="48"/>
     </x:row>
-    <x:row r="99" ht="46" customHeight="1">
+    <x:row r="99" ht="72" customHeight="1">
       <x:c r="A99" s="48" t="str">
         <x:v>TG-0570</x:v>
       </x:c>
@@ -12339,7 +12339,7 @@
         <x:v>«Википедия» считает, что одна ОНА больше известна под фамилией Белобородова. МОК аннулировал ее золотую медаль Олимпиады-2012. Другая ОНА имела непосредственное отношение к интеллектуальным играм, но стала известной благодаря спортивным медиа. ОН - один из самых заметных и известных журналистов «Чемпионата». Какая фамилия объединяет этих людей?</x:v>
       </x:c>
       <x:c r="E99" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Лысенко</x:v>
       </x:c>
       <x:c r="F99" s="50" t="str">
         <x:v>https://t.me/simple_quiz/570</x:v>
@@ -12351,11 +12351,11 @@
         <x:v>0.9488</x:v>
       </x:c>
       <x:c r="I99" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J99" s="48"/>
     </x:row>
-    <x:row r="100" ht="46" customHeight="1">
+    <x:row r="100" ht="72" customHeight="1">
       <x:c r="A100" s="48" t="str">
         <x:v>TG-0571</x:v>
       </x:c>
@@ -12385,7 +12385,7 @@
       </x:c>
       <x:c r="J100" s="48"/>
     </x:row>
-    <x:row r="101" ht="46" customHeight="1">
+    <x:row r="101" ht="72" customHeight="1">
       <x:c r="A101" s="48" t="str">
         <x:v>TG-0572</x:v>
       </x:c>
@@ -12399,7 +12399,7 @@
         <x:v>50 Cent - 21 ИКС. Обладатель второго места конкурса комментаторов «России-2» в 2012 году - 50 ИКСОВ. Чему равен ИКС?</x:v>
       </x:c>
       <x:c r="E101" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Вопрос (question)</x:v>
       </x:c>
       <x:c r="F101" s="50" t="str">
         <x:v>https://t.me/simple_quiz/572</x:v>
@@ -12411,11 +12411,11 @@
         <x:v>0.9431</x:v>
       </x:c>
       <x:c r="I101" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J101" s="48"/>
     </x:row>
-    <x:row r="102" ht="46" customHeight="1">
+    <x:row r="102" ht="72" customHeight="1">
       <x:c r="A102" s="48" t="str">
         <x:v>TG-0587</x:v>
       </x:c>
@@ -12429,7 +12429,7 @@
         <x:v>В пьесе «Двенадцатая ночь» Уильям Шекспир писал, что дурацкий колпак ПРОПУСК не портит. ПРОПУСК точно не испортил «Кливленд» в 2016 году, ведь команда стала чемпионом НБА. Восполните ПРОПУСК.</x:v>
       </x:c>
       <x:c r="E102" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Мозгов</x:v>
       </x:c>
       <x:c r="F102" s="50" t="str">
         <x:v>https://t.me/simple_quiz/587</x:v>
@@ -12441,11 +12441,11 @@
         <x:v>0.9624</x:v>
       </x:c>
       <x:c r="I102" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J102" s="48"/>
     </x:row>
-    <x:row r="103" ht="46" customHeight="1">
+    <x:row r="103" ht="72" customHeight="1">
       <x:c r="A103" s="48" t="str">
         <x:v>TG-0588</x:v>
       </x:c>
@@ -12459,7 +12459,7 @@
         <x:v>Матч «Арсенала» и «Кристал Пэласа» 1 января 2017 года вызвал много шуток и реакций в соцсетях и на спортивных сайтах из-за ЕГО гола: русскоязычные фанаты футбола посчитали ЕГО гол довольно символичным. Кто забил гол в том матче?</x:v>
       </x:c>
       <x:c r="E103" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Оливье Жиру</x:v>
       </x:c>
       <x:c r="F103" s="50" t="str">
         <x:v>https://t.me/simple_quiz/588</x:v>
@@ -12471,11 +12471,11 @@
         <x:v>0.9576</x:v>
       </x:c>
       <x:c r="I103" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J103" s="48"/>
     </x:row>
-    <x:row r="104" ht="46" customHeight="1">
+    <x:row r="104" ht="72" customHeight="1">
       <x:c r="A104" s="48" t="str">
         <x:v>TG-0589</x:v>
       </x:c>
@@ -12489,7 +12489,7 @@
         <x:v>ОН на английском - бывший футболист, забивавший за «Лацио» и «Рейнджерс». ОН на русском - главный герой мультфильма «Пес в сапогах». Назовите ЕГО по-английски или по-русски.</x:v>
       </x:c>
       <x:c r="E104" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Gascoigne / Гасконец</x:v>
       </x:c>
       <x:c r="F104" s="50" t="str">
         <x:v>https://t.me/simple_quiz/589</x:v>
@@ -12501,11 +12501,11 @@
         <x:v>0.9447</x:v>
       </x:c>
       <x:c r="I104" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J104" s="48"/>
     </x:row>
-    <x:row r="105" ht="46" customHeight="1">
+    <x:row r="105" ht="72" customHeight="1">
       <x:c r="A105" s="48" t="str">
         <x:v>TG-0594</x:v>
       </x:c>
@@ -12519,7 +12519,7 @@
         <x:v>Жительница Манилы четыре года молилась статуэтке ИКСА, ошибочно думая, что это Хотэй - популярное в китайской культуре божество счастья, благополучия, веселья и общения. Ее смутил большой живот статуэтки. ИКС — прозвище футболиста, который по завершении карьеры потренировал клубы из Вашингтона, Плимута, Бирмингема и Дерби. Назовите ИКС.</x:v>
       </x:c>
       <x:c r="E105" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Шрек</x:v>
       </x:c>
       <x:c r="F105" s="50" t="str">
         <x:v>https://t.me/simple_quiz/594</x:v>
@@ -12531,11 +12531,11 @@
         <x:v>0.9422</x:v>
       </x:c>
       <x:c r="I105" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J105" s="48"/>
     </x:row>
-    <x:row r="106" ht="46" customHeight="1">
+    <x:row r="106" ht="72" customHeight="1">
       <x:c r="A106" s="48" t="str">
         <x:v>TG-0601</x:v>
       </x:c>
@@ -12549,7 +12549,7 @@
         <x:v>На альбоме «Пиры и раны» группы «Кровосток» есть песна «ЗАМЕНА». ЗАМЕНА состоит из двух глаголов, которые образуют фразу, используемую для ироничного описания тактики некоторых футбольных команд. ЗАМЕНА - правда, с чуть измененной орфографией, — название ныне несуществующей медиафутбольной команды. Воспроизведите ЗАМЕНУ.</x:v>
       </x:c>
       <x:c r="E106" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Бей-беги</x:v>
       </x:c>
       <x:c r="F106" s="50" t="str">
         <x:v>https://t.me/simple_quiz/601</x:v>
@@ -12561,11 +12561,11 @@
         <x:v>0.9477</x:v>
       </x:c>
       <x:c r="I106" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J106" s="48"/>
     </x:row>
-    <x:row r="107" ht="46" customHeight="1">
+    <x:row r="107" ht="72" customHeight="1">
       <x:c r="A107" s="48" t="str">
         <x:v>TG-0604</x:v>
       </x:c>
@@ -12579,7 +12579,7 @@
         <x:v>Сайт 9meters подсчитал, что в мире живет 2700 ТАКИХ людей. 33 из 2700 ТАКИХ людей играют в НБА. ТАКИЕ - составное прилагательное, причем второй корень очень редко используется в России и часто — в США. Что мы зашифровали под ТАКИМИ?</x:v>
       </x:c>
       <x:c r="E107" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Семифутеры</x:v>
       </x:c>
       <x:c r="F107" s="50" t="str">
         <x:v>https://t.me/simple_quiz/604</x:v>
@@ -12591,11 +12591,11 @@
         <x:v>0.9475</x:v>
       </x:c>
       <x:c r="I107" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J107" s="48"/>
     </x:row>
-    <x:row r="108" ht="46" customHeight="1">
+    <x:row r="108" ht="72" customHeight="1">
       <x:c r="A108" s="48" t="str">
         <x:v>TG-0607</x:v>
       </x:c>
@@ -12609,7 +12609,7 @@
         <x:v>АЛЬФОЙ в славянской мифологии называли духа умершего человека в облике женщины. Известная вам АЛЬФА - олимпийская чемпионка, которая сначала вышла замуж за тренера, а затем — за человека, в честь отличительной особенности которого назвали либеральное микромедиа. Назовите АЛЬФУ.</x:v>
       </x:c>
       <x:c r="E108" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Навка</x:v>
       </x:c>
       <x:c r="F108" s="50" t="str">
         <x:v>https://t.me/simple_quiz/607</x:v>
@@ -12621,11 +12621,11 @@
         <x:v>0.9517</x:v>
       </x:c>
       <x:c r="I108" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J108" s="48"/>
     </x:row>
-    <x:row r="109" ht="46" customHeight="1">
+    <x:row r="109" ht="72" customHeight="1">
       <x:c r="A109" s="48" t="str">
         <x:v>TG-0611</x:v>
       </x:c>
@@ -12639,7 +12639,7 @@
         <x:v>Поговорим о маршрутах. Из «Селтикс» в «Суперсоникс» - 90. Из «Селтикс» в «Уорриорз» - 80. Из «Уизардс» в «Уорриорз» - 50. Число, которое соответствует маршруту Пау Газоля в 2014-м, вы прекрасно знаете: ему посвящено много отсылок в поп-культуре. Назовите его.</x:v>
       </x:c>
       <x:c r="E109" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Route 66</x:v>
       </x:c>
       <x:c r="F109" s="50" t="str">
         <x:v>https://t.me/simple_quiz/611</x:v>
@@ -12651,11 +12651,11 @@
         <x:v>0.9447</x:v>
       </x:c>
       <x:c r="I109" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J109" s="48"/>
     </x:row>
-    <x:row r="110" ht="46" customHeight="1">
+    <x:row r="110" ht="72" customHeight="1">
       <x:c r="A110" s="48" t="str">
         <x:v>TG-0613</x:v>
       </x:c>
@@ -12669,7 +12669,7 @@
         <x:v>Если бы популярный российский блогер получил прозвище, потому что он EE сын, это было бы намного более логично. Но нет: несмотря на совпадение фамилий, он не состоит с НЕЙ в родственных связях. ОНА завоевала серебряную медаль на ОИ в Сиднее и сразу две медали - золото и бронзу - в Афинах. Назовите EE имя и фамилию.</x:v>
       </x:c>
       <x:c r="E110" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Татьяна Лебедева</x:v>
       </x:c>
       <x:c r="F110" s="50" t="str">
         <x:v>https://t.me/simple_quiz/613</x:v>
@@ -12681,11 +12681,11 @@
         <x:v>0.9554</x:v>
       </x:c>
       <x:c r="I110" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J110" s="48"/>
     </x:row>
-    <x:row r="111" ht="46" customHeight="1">
+    <x:row r="111" ht="72" customHeight="1">
       <x:c r="A111" s="48" t="str">
         <x:v>TG-0617</x:v>
       </x:c>
@@ -12699,7 +12699,7 @@
         <x:v>Один ОН - французский автогонщик, девятикратный чемпион мира. Другой ОН - немецкий автогонщик, четырехкратный чемпион мира. Было бы символично, если бы и первый, и второй ОН одержали победы в одном испанском городе, но гонки, в которых они принимали участие, в нем не проходили. Назовите ЕГО.</x:v>
       </x:c>
       <x:c r="E111" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Сан-Себастьян</x:v>
       </x:c>
       <x:c r="F111" s="50" t="str">
         <x:v>https://t.me/simple_quiz/617</x:v>
@@ -12711,11 +12711,11 @@
         <x:v>0.9494</x:v>
       </x:c>
       <x:c r="I111" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J111" s="48"/>
     </x:row>
-    <x:row r="112" ht="46" customHeight="1">
+    <x:row r="112" ht="72" customHeight="1">
       <x:c r="A112" s="48" t="str">
         <x:v>TG-0618</x:v>
       </x:c>
@@ -12729,7 +12729,7 @@
         <x:v>1988, 1992, 1996, 2000 - ПЕРВЫЕ. 1988, 1992, 1994, 1998 —- ВТОРЫЕ. Назовите ПЕРВЫЕ и ВТОРЫЕ.</x:v>
       </x:c>
       <x:c r="E112" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Летние и зимние Олимпийские игры</x:v>
       </x:c>
       <x:c r="F112" s="50" t="str">
         <x:v>https://t.me/simple_quiz/618</x:v>
@@ -12741,11 +12741,11 @@
         <x:v>0.9302</x:v>
       </x:c>
       <x:c r="I112" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J112" s="48"/>
     </x:row>
-    <x:row r="113" ht="46" customHeight="1">
+    <x:row r="113" ht="72" customHeight="1">
       <x:c r="A113" s="48" t="str">
         <x:v>TG-0620</x:v>
       </x:c>
@@ -12759,7 +12759,7 @@
         <x:v>«Манчестер Сити», «Интер», «Лилль», «Бавария», «Атлетико» - все эти клубы объединяет трек FRIENDLY THUG 52 МСС с альбома «Graf Monte-Cristo/Most Valuable Pirate». Воспроизведите название этого трека.</x:v>
       </x:c>
       <x:c r="E113" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F113" s="50" t="str">
         <x:v>https://t.me/simple_quiz/620</x:v>
@@ -12771,11 +12771,11 @@
         <x:v>0.9527</x:v>
       </x:c>
       <x:c r="I113" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J113" s="48"/>
     </x:row>
-    <x:row r="114" ht="46" customHeight="1">
+    <x:row r="114" ht="72" customHeight="1">
       <x:c r="A114" s="48" t="str">
         <x:v>TG-0623</x:v>
       </x:c>
@@ -12789,7 +12789,7 @@
         <x:v>В интернете можно найти победителей ЭТОГО турнира с 1949 года. Вот некоторые из них. 2025 - Джексон Шторм. 2024 - Пол Корнев. 2023 - Райан Лэйни. 2022 - Тим Тредлесс. 2021 - Круз Рамирес. 2020 - Чейз Рейселотт. В 2006, 2007, 2009, 2010, 2011, 2012 и 2015 годах победителем становился рекордсмен, которому даже посвятили серию фильмов. Назовите турнир, о котором идет речь.</x:v>
       </x:c>
       <x:c r="E114" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Кубок Поршня</x:v>
       </x:c>
       <x:c r="F114" s="50" t="str">
         <x:v>https://t.me/simple_quiz/623</x:v>
@@ -12801,11 +12801,11 @@
         <x:v>0.9395</x:v>
       </x:c>
       <x:c r="I114" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J114" s="48"/>
     </x:row>
-    <x:row r="115" ht="46" customHeight="1">
+    <x:row r="115" ht="72" customHeight="1">
       <x:c r="A115" s="48" t="str">
         <x:v>TG-0624</x:v>
       </x:c>
@@ -12819,7 +12819,7 @@
         <x:v>В английском языке для того, чтобы превратить фамилию главного героя культового сериала в фамилию члена Зала славы снукера, необходимо убрать согласную букву. В русском языке для того, чтобы превратить фамилию главного героя культового сериала в фамилию члена Зала славы снукера, необходимо заменить согласную букву. Назовите члена Зала славы снукера, о котором идет речь.</x:v>
       </x:c>
       <x:c r="E115" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Марк Селби</x:v>
       </x:c>
       <x:c r="F115" s="50" t="str">
         <x:v>https://t.me/simple_quiz/624</x:v>
@@ -12831,11 +12831,11 @@
         <x:v>0.9591</x:v>
       </x:c>
       <x:c r="I115" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J115" s="48"/>
     </x:row>
-    <x:row r="116" ht="46" customHeight="1">
+    <x:row r="116" ht="72" customHeight="1">
       <x:c r="A116" s="48" t="str">
         <x:v>TG-0625</x:v>
       </x:c>
@@ -12849,7 +12849,7 @@
         <x:v>Обидно, что в «Орландо» нет футболиста по имени и фамилии Эйбел - они бы составили потрясающую, чуть ли не братскую связку с другим игроком «Мэджик». Назовите фамилию этого игрока - или ее русскоязычный аналог.</x:v>
       </x:c>
       <x:c r="E116" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Каин</x:v>
       </x:c>
       <x:c r="F116" s="50" t="str">
         <x:v>https://t.me/simple_quiz/625</x:v>
@@ -12861,11 +12861,11 @@
         <x:v>0.9531</x:v>
       </x:c>
       <x:c r="I116" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J116" s="48"/>
     </x:row>
-    <x:row r="117" ht="46" customHeight="1">
+    <x:row r="117" ht="72" customHeight="1">
       <x:c r="A117" s="48" t="str">
         <x:v>TG-0628</x:v>
       </x:c>
@@ -12879,7 +12879,7 @@
         <x:v>Баскетболист «Никс» Карл-Энтони Таунс приехал на Матч звезд НБА в бомбере, на спине которого был изображен христианский святой в узнаваемом образе. Согласно житию этого святого, он родился в Каппадокии. А его изображение вы точно видели много раз. Возможно, вам помогут догадаться, где оно вам встречалось, числа 1, 5, 10 и 50. Назовите этого святого двумя словами.</x:v>
       </x:c>
       <x:c r="E117" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Георгий Победоносец</x:v>
       </x:c>
       <x:c r="F117" s="50" t="str">
         <x:v>https://t.me/simple_quiz/628</x:v>
@@ -12891,11 +12891,11 @@
         <x:v>0.9471</x:v>
       </x:c>
       <x:c r="I117" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J117" s="48"/>
     </x:row>
-    <x:row r="118" ht="46" customHeight="1">
+    <x:row r="118" ht="72" customHeight="1">
       <x:c r="A118" s="48" t="str">
         <x:v>TG-0635</x:v>
       </x:c>
@@ -12927,7 +12927,7 @@
         <x:v>38</x:v>
       </x:c>
     </x:row>
-    <x:row r="119" ht="46" customHeight="1">
+    <x:row r="119" ht="72" customHeight="1">
       <x:c r="A119" s="48" t="str">
         <x:v>TG-0636</x:v>
       </x:c>
@@ -12959,7 +12959,7 @@
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="120" ht="46" customHeight="1">
+    <x:row r="120" ht="72" customHeight="1">
       <x:c r="A120" s="48" t="str">
         <x:v>TG-0644</x:v>
       </x:c>
@@ -12991,7 +12991,7 @@
         <x:v>27</x:v>
       </x:c>
     </x:row>
-    <x:row r="121" ht="46" customHeight="1">
+    <x:row r="121" ht="72" customHeight="1">
       <x:c r="A121" s="48" t="str">
         <x:v>TG-0645</x:v>
       </x:c>
@@ -13023,7 +13023,7 @@
         <x:v>23</x:v>
       </x:c>
     </x:row>
-    <x:row r="122" ht="46" customHeight="1">
+    <x:row r="122" ht="72" customHeight="1">
       <x:c r="A122" s="48" t="str">
         <x:v>TG-0647</x:v>
       </x:c>
@@ -13055,7 +13055,7 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="123" ht="46" customHeight="1">
+    <x:row r="123" ht="72" customHeight="1">
       <x:c r="A123" s="48" t="str">
         <x:v>TG-0648</x:v>
       </x:c>
@@ -13087,7 +13087,7 @@
         <x:v>12</x:v>
       </x:c>
     </x:row>
-    <x:row r="124" ht="46" customHeight="1">
+    <x:row r="124" ht="72" customHeight="1">
       <x:c r="A124" s="48" t="str">
         <x:v>TG-0649</x:v>
       </x:c>
@@ -13119,7 +13119,7 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="125" ht="46" customHeight="1">
+    <x:row r="125" ht="72" customHeight="1">
       <x:c r="A125" s="48" t="str">
         <x:v>TG-0659</x:v>
       </x:c>
@@ -13151,7 +13151,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="126" ht="46" customHeight="1">
+    <x:row r="126" ht="72" customHeight="1">
       <x:c r="A126" s="48" t="str">
         <x:v>TG-0664</x:v>
       </x:c>
@@ -13165,7 +13165,7 @@
         <x:v>В 2021 году Леонид Слуцкий сделал ЕЕ: он рассказал об этом Ксении Собчак на ее УочТиБе-канале. С 2022 года многие россияне начали намного чаще делать EE, если хотят посетить страны Европы, Азии и Америки. Назовите EE тремя словами.</x:v>
       </x:c>
       <x:c r="E126" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Пересадка в Турции</x:v>
       </x:c>
       <x:c r="F126" s="50" t="str">
         <x:v>https://t.me/simple_quiz/664</x:v>
@@ -13177,11 +13177,11 @@
         <x:v>0.9532</x:v>
       </x:c>
       <x:c r="I126" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J126" s="48"/>
     </x:row>
-    <x:row r="127" ht="46" customHeight="1">
+    <x:row r="127" ht="72" customHeight="1">
       <x:c r="A127" s="48" t="str">
         <x:v>TG-0669</x:v>
       </x:c>
@@ -13195,7 +13195,7 @@
         <x:v>Один из экспертов по русскому футболу дал такую характеристику 20-летнему форварду «Уфы» и воспитаннику одного из топ-клубов РПЛ Алексею Барановскому: «Он наглый пацан, который хорошо умеет играть в футбол. Говорю ему: все отлично, кроме фамилии». Назовите эксперта, который дал эту характеристику.</x:v>
       </x:c>
       <x:c r="E127" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Андрей Аршавин</x:v>
       </x:c>
       <x:c r="F127" s="50" t="str">
         <x:v>https://t.me/simple_quiz/669</x:v>
@@ -13207,11 +13207,11 @@
         <x:v>0.9577</x:v>
       </x:c>
       <x:c r="I127" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J127" s="48"/>
     </x:row>
-    <x:row r="128" ht="46" customHeight="1">
+    <x:row r="128" ht="72" customHeight="1">
       <x:c r="A128" s="48" t="str">
         <x:v>TG-0682</x:v>
       </x:c>
@@ -13225,7 +13225,7 @@
         <x:v>Перед вами фрагмент постера, со Ма та посвященного одному =. м. ее спортивному событию. Горы, rh. которые стали частью Ч 4 а композиции, мы скрыли. AS ; Мы He спрашиваем вас, что А . это за событие - напишите, в 12 форме чего выполнен силуэт Ni города на этом постере. (5 R E</x:v>
       </x:c>
       <x:c r="E128" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Олимпийский факел</x:v>
       </x:c>
       <x:c r="F128" s="50" t="str">
         <x:v>https://t.me/simple_quiz/682</x:v>
@@ -13237,11 +13237,11 @@
         <x:v>0.7423</x:v>
       </x:c>
       <x:c r="I128" s="50" t="str">
-        <x:v>OCR — проверить формулировку</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J128" s="48"/>
     </x:row>
-    <x:row r="129" ht="46" customHeight="1">
+    <x:row r="129" ht="72" customHeight="1">
       <x:c r="A129" s="48" t="str">
         <x:v>TG-0684</x:v>
       </x:c>
@@ -13255,7 +13255,7 @@
         <x:v>Обратная ОНА была распространенным приемом в византийской и древнерусской иконописи. Когда речь идет о талантливых спортсменах, часто говорят о НЕЙ и называют ТАКИМИ - прилагательным, образованным от слова ОНА. Правда, чем старше спортсмен, тем реже мы говорим о том, что он - ТАКОЙ. Даи ИХ у него становится меньше. Назовите EE.</x:v>
       </x:c>
       <x:c r="E129" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Перспектива</x:v>
       </x:c>
       <x:c r="F129" s="50" t="str">
         <x:v>https://t.me/simple_quiz/684</x:v>
@@ -13267,11 +13267,11 @@
         <x:v>0.955</x:v>
       </x:c>
       <x:c r="I129" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J129" s="48"/>
     </x:row>
-    <x:row r="130" ht="46" customHeight="1">
+    <x:row r="130" ht="72" customHeight="1">
       <x:c r="A130" s="48" t="str">
         <x:v>TG-0716</x:v>
       </x:c>
@@ -13301,7 +13301,7 @@
       </x:c>
       <x:c r="J130" s="48"/>
     </x:row>
-    <x:row r="131" ht="46" customHeight="1">
+    <x:row r="131" ht="72" customHeight="1">
       <x:c r="A131" s="48" t="str">
         <x:v>TG-0717</x:v>
       </x:c>
@@ -13315,7 +13315,7 @@
         <x:v>Несмотря на то, что эта европейская страна не попала на чемпионат мира по футболу, ее англоязычное название можно было увидеть во время трансляций как минимум восьми матчей ЧМ-2026. Назовите эту европейскую страну.</x:v>
       </x:c>
       <x:c r="E131" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Грузия</x:v>
       </x:c>
       <x:c r="F131" s="50" t="str">
         <x:v>https://t.me/simple_quiz/717</x:v>
@@ -13327,11 +13327,11 @@
         <x:v>0.9595</x:v>
       </x:c>
       <x:c r="I131" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J131" s="48"/>
     </x:row>
-    <x:row r="132" ht="46" customHeight="1">
+    <x:row r="132" ht="72" customHeight="1">
       <x:c r="A132" s="48" t="str">
         <x:v>TG-0718</x:v>
       </x:c>
@@ -13345,7 +13345,7 @@
         <x:v>В 2006 году на платформе PSP вышла игра, где основной механикой был наклон планеты. Первая часть названия - испанское слово, которое совпадает с прозвищем тренера, не вышедшего вместе со сборной из группы на ЧМ-2026. Назовите фамилию этого тренера.</x:v>
       </x:c>
       <x:c r="E132" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Марсело Бьельса</x:v>
       </x:c>
       <x:c r="F132" s="50" t="str">
         <x:v>https://t.me/simple_quiz/718</x:v>
@@ -13357,11 +13357,11 @@
         <x:v>0.957</x:v>
       </x:c>
       <x:c r="I132" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён реакцией канала</x:v>
       </x:c>
       <x:c r="J132" s="48"/>
     </x:row>
-    <x:row r="133" ht="46" customHeight="1">
+    <x:row r="133" ht="72" customHeight="1">
       <x:c r="A133" s="48" t="str">
         <x:v>TG-0719</x:v>
       </x:c>
@@ -13403,12 +13403,12 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="I4:I133">
-      <x:formula1>"Распознано — проверить ответ,OCR — проверить формулировку,Дубликат каталога,Проверено"</x:formula1>
+      <x:formula1>"Распознано — проверить ответ,OCR — проверить формулировку,Дубликат каталога,Ответ подтверждён реакцией канала,Проверено"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ccd4ea635df4fa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24abddc24cd43f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct answer for catalog question 53
</commit_message>
<xml_diff>
--- a/Simple_Quiz_Intelligence_v1_rebuilt.xlsx
+++ b/Simple_Quiz_Intelligence_v1_rebuilt.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Каталог" sheetId="1" r:id="R2fc779dd31c543cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Механики" sheetId="2" r:id="Re8647745720143a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Раунды" sheetId="3" r:id="R195218a2d7fe47bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дашборд" sheetId="4" r:id="Rc8b75b4f86b44b76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Новые пакеты" sheetId="5" r:id="R8e8e1aedc90242b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram-архив" sheetId="6" r:id="Rca472f345e024a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Каталог" sheetId="1" r:id="Reb02543238f24fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Механики" sheetId="2" r:id="Rfecdde80cd6144d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Раунды" sheetId="3" r:id="R365ab78999be4969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дашборд" sheetId="4" r:id="R857a10b2a9214800"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Новые пакеты" sheetId="5" r:id="R38701e2805f74ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram-архив" sheetId="6" r:id="R7bff7c2e620448b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -426,7 +426,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdfbec3e15ba947cf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f00b371ac584528"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3068,7 +3068,7 @@
         <x:v>В одной легендарной московской команде середины 2000-х было два русских спортсмена с редко встречающимися фамилиями. Одна из них дословно означает пузо или желудок. Другая - верхние листы кочана капусты. Впоследствии оба поиграли на другом материке, но доигрывали последние годы карьеры в российских клубах. Назовите фамилии этих спортсменов.</x:v>
       </x:c>
       <x:c r="F54" s="7" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Моня и Хряпа</x:v>
       </x:c>
       <x:c r="G54" s="7" t="str">
         <x:v>Не размечено</x:v>
@@ -3077,7 +3077,7 @@
         <x:v>Спорт / смешанное</x:v>
       </x:c>
       <x:c r="I54" s="7" t="str">
-        <x:v>OCR из карточки; требуется редакторская проверка</x:v>
+        <x:v>Ответ уточнён пользователем: Уточнение пользователя</x:v>
       </x:c>
       <x:c r="J54" s="6"/>
       <x:c r="K54" s="6" t="str">
@@ -7791,7 +7791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4777c06e4b5047c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2a34146de4949cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8467,7 +8467,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefd9b9808a541f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ba20e606fa14f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8639,7 +8639,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6631473d2eb847c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ea5bde8468240fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8903,7 +8903,7 @@
     <x:mergeCell ref="E9:H9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58654fc5740548a6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2369298a080040de"/>
 </x:worksheet>
 </file>
 
@@ -9394,7 +9394,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb22a28fec224528"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f4e9bc38e8c4c23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9431,7 +9431,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="44" t="str">
-        <x:v>130 распознанных карточек; 122 новых вопросов добавлено в «Каталог», 8 совпадений отмечено как дубликаты. 113 ответов заполнено.</x:v>
+        <x:v>130 распознанных карточек; 122 новых вопросов добавлено в «Каталог», 8 совпадений отмечено как дубликаты. 114 ответов заполнено.</x:v>
       </x:c>
       <x:c r="B2" s="44"/>
       <x:c r="C2" s="44"/>
@@ -9609,7 +9609,7 @@
         <x:v>В одной легендарной московской команде середины 2000-х было два русских спортсмена с редко встречающимися фамилиями. Одна из них дословно означает пузо или желудок. Другая - верхние листы кочана капусты. Впоследствии оба поиграли на другом материке, но доигрывали последние годы карьеры в российских клубах. Назовите фамилии этих спортсменов.</x:v>
       </x:c>
       <x:c r="E8" s="50" t="str">
-        <x:v>Не опубликован в посте</x:v>
+        <x:v>Моня и Хряпа</x:v>
       </x:c>
       <x:c r="F8" s="50" t="str">
         <x:v>https://t.me/simple_quiz/35</x:v>
@@ -9621,7 +9621,7 @@
         <x:v>0.9536</x:v>
       </x:c>
       <x:c r="I8" s="50" t="str">
-        <x:v>Распознано — проверить ответ</x:v>
+        <x:v>Ответ подтверждён пользователем</x:v>
       </x:c>
       <x:c r="J8" s="48"/>
     </x:row>
@@ -13403,12 +13403,12 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="I4:I133">
-      <x:formula1>"Распознано — проверить ответ,OCR — проверить формулировку,Дубликат каталога,Ответ подтверждён реакцией канала,Проверено"</x:formula1>
+      <x:formula1>"Распознано — проверить ответ,OCR — проверить формулировку,Дубликат каталога,Ответ подтверждён реакцией канала,Ответ подтверждён пользователем,Проверено"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24abddc24cd43f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d1a13b730df479d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>